<commit_message>
Added Respawning, spawn class for enemies, health changing to BP_Player, death zone, checkpoints, health pickup, and changed test level.
</commit_message>
<xml_diff>
--- a/Red Team Tracebility and Testing.xlsx
+++ b/Red Team Tracebility and Testing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Program Files\Epic Games\UE_5.7\redteam\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03847EFE-33D6-4DAA-837E-6436BDAB8B46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD5AE3FF-7369-4349-92CA-CA37A00F6F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{19EF330C-6F54-4365-A47E-10806019DE9B}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Test Plan" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Traceability Matrix'!$G$5:$G$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Traceability Matrix'!$H$5:$H$37</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="146">
   <si>
     <t>Prototype Title:</t>
   </si>
@@ -377,9 +377,6 @@
     <t>Add Controls that moves player horizontally using A and D.</t>
   </si>
   <si>
-    <t>Need to decide on checkpoint placement…</t>
-  </si>
-  <si>
     <t>Traceability Matrix (Red Team)</t>
   </si>
   <si>
@@ -519,13 +516,64 @@
   </si>
   <si>
     <t>William Meredith (5:47PM, 5/23/2026)</t>
+  </si>
+  <si>
+    <t>Added player Health Pickups with a  temp heart model. -Nathen Reed</t>
+  </si>
+  <si>
+    <t>Checkpoints added with temp Placeholder. -Nathen Reed</t>
+  </si>
+  <si>
+    <t>Big deathzone added that resets player to respawn point. -Nathen Reed</t>
+  </si>
+  <si>
+    <t>Added accurate collision to current Tilesets.</t>
+  </si>
+  <si>
+    <t>Player Not getting teleported.</t>
+  </si>
+  <si>
+    <t>Received errors from respawn event due to the variable used for the spawn transform coming in empty.</t>
+  </si>
+  <si>
+    <t>Error was caused by player not being passed with the call to the RespawnEvent. Ensuring this was hooked in properly fixed the error.</t>
+  </si>
+  <si>
+    <t>Nathen Reed (5:39PM, 5/31/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carrot: Ranged, Feather: Double Jump, Arrow: Dash? </t>
+  </si>
+  <si>
+    <t>Jump attack placed within enemy classes.  -Nathen Reed</t>
+  </si>
+  <si>
+    <t>Added 1 second shield upon damage -Nathen Reed</t>
+  </si>
+  <si>
+    <t>Health Pickup</t>
+  </si>
+  <si>
+    <t>Health Pickup design</t>
+  </si>
+  <si>
+    <t>Temp floating heart added by Nathen Reed. -Nathen Reed</t>
+  </si>
+  <si>
+    <t>Rabbit Player model added with flipbook</t>
+  </si>
+  <si>
+    <t>Coins</t>
+  </si>
+  <si>
+    <t>Collectable coins they stay tracked on UI.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -565,13 +613,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <i/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -752,7 +793,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="39">
+  <borders count="38">
     <border>
       <left/>
       <right/>
@@ -1043,59 +1084,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color indexed="64"/>
@@ -1220,25 +1208,73 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="124">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
@@ -1246,7 +1282,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1264,9 +1300,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1292,55 +1325,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1349,110 +1364,170 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1460,106 +1535,61 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1882,7 +1912,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB4A1F4-D2AB-4474-B05F-C8B13F4E557C}">
-  <dimension ref="A1:AC35"/>
+  <dimension ref="A1:AC38"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" style="1" customWidth="1"/>
@@ -1898,30 +1928,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="105" t="s">
-        <v>83</v>
-      </c>
-      <c r="B1" s="106"/>
-      <c r="C1" s="106"/>
-      <c r="D1" s="106"/>
-      <c r="E1" s="106"/>
-      <c r="F1" s="106"/>
-      <c r="G1" s="106"/>
-      <c r="H1" s="106"/>
-      <c r="I1" s="106"/>
+      <c r="A1" s="84" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="85"/>
+      <c r="C1" s="85"/>
+      <c r="D1" s="85"/>
+      <c r="E1" s="85"/>
+      <c r="F1" s="85"/>
+      <c r="G1" s="85"/>
+      <c r="H1" s="85"/>
+      <c r="I1" s="85"/>
     </row>
     <row r="2" spans="1:29" s="3" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="102"/>
-      <c r="C2" s="103"/>
-      <c r="D2" s="103"/>
-      <c r="E2" s="103"/>
-      <c r="F2" s="103"/>
-      <c r="G2" s="103"/>
-      <c r="H2" s="103"/>
-      <c r="I2" s="104"/>
+      <c r="B2" s="81"/>
+      <c r="C2" s="82"/>
+      <c r="D2" s="82"/>
+      <c r="E2" s="82"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="82"/>
+      <c r="H2" s="82"/>
+      <c r="I2" s="83"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
@@ -1940,90 +1970,90 @@
       <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="107" t="s">
-        <v>85</v>
-      </c>
-      <c r="C3" s="108"/>
-      <c r="D3" s="108"/>
-      <c r="E3" s="108"/>
-      <c r="F3" s="108"/>
-      <c r="G3" s="108"/>
-      <c r="H3" s="108"/>
-      <c r="I3" s="109"/>
+      <c r="B3" s="86" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="87"/>
+      <c r="D3" s="87"/>
+      <c r="E3" s="87"/>
+      <c r="F3" s="87"/>
+      <c r="G3" s="87"/>
+      <c r="H3" s="87"/>
+      <c r="I3" s="88"/>
     </row>
     <row r="4" spans="1:29" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="45" t="s">
-        <v>84</v>
-      </c>
-      <c r="B4" s="110" t="s">
-        <v>87</v>
-      </c>
-      <c r="C4" s="111"/>
-      <c r="D4" s="111"/>
-      <c r="E4" s="111"/>
-      <c r="F4" s="111"/>
-      <c r="G4" s="111"/>
-      <c r="H4" s="111"/>
-      <c r="I4" s="112"/>
+      <c r="A4" s="38" t="s">
+        <v>83</v>
+      </c>
+      <c r="B4" s="89" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" s="90"/>
+      <c r="D4" s="90"/>
+      <c r="E4" s="90"/>
+      <c r="F4" s="90"/>
+      <c r="G4" s="90"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="91"/>
     </row>
     <row r="5" spans="1:29" s="2" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="77" t="s">
+      <c r="A5" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="77" t="s">
+      <c r="B5" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="77" t="s">
+      <c r="C5" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="77" t="s">
+      <c r="D5" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="77" t="s">
+      <c r="E5" s="63" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="77" t="s">
+      <c r="F5" s="63" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="77" t="s">
+      <c r="G5" s="63" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="42" t="s">
+      <c r="H5" s="35" t="s">
         <v>58</v>
       </c>
-      <c r="I5" s="42" t="s">
-        <v>90</v>
+      <c r="I5" s="35" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:29" s="8" customFormat="1" ht="46.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="116" t="s">
+      <c r="A6" s="95" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="79" t="s">
+      <c r="B6" s="65" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="80" t="s">
+      <c r="C6" s="66" t="s">
         <v>81</v>
       </c>
-      <c r="D6" s="80" t="s">
+      <c r="D6" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="59" t="s">
+      <c r="E6" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="60" t="s">
+      <c r="F6" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="81" t="s">
-        <v>96</v>
-      </c>
-      <c r="H6" s="86" t="s">
+      <c r="G6" s="67" t="s">
+        <v>95</v>
+      </c>
+      <c r="H6" s="72" t="s">
+        <v>114</v>
+      </c>
+      <c r="I6" s="73" t="s">
         <v>115</v>
       </c>
-      <c r="I6" s="87" t="s">
-        <v>116</v>
-      </c>
-      <c r="J6" s="21"/>
+      <c r="J6" s="20"/>
       <c r="K6"/>
       <c r="L6"/>
       <c r="M6"/>
@@ -2045,8 +2075,8 @@
       <c r="AC6"/>
     </row>
     <row r="7" spans="1:29" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="117"/>
-      <c r="B7" s="82" t="s">
+      <c r="A7" s="96"/>
+      <c r="B7" s="68" t="s">
         <v>51</v>
       </c>
       <c r="C7" s="9" t="s">
@@ -2055,46 +2085,48 @@
       <c r="D7" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="43" t="s">
-        <v>92</v>
-      </c>
-      <c r="F7" s="43" t="s">
+      <c r="E7" s="36" t="s">
+        <v>91</v>
+      </c>
+      <c r="F7" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="83" t="s">
-        <v>96</v>
-      </c>
-      <c r="H7" s="64" t="s">
+      <c r="G7" s="69" t="s">
+        <v>95</v>
+      </c>
+      <c r="H7" s="107" t="s">
+        <v>114</v>
+      </c>
+      <c r="I7" s="120" t="s">
+        <v>139</v>
+      </c>
+      <c r="J7" s="20"/>
+    </row>
+    <row r="8" spans="1:29" s="7" customFormat="1" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="97"/>
+      <c r="B8" s="51" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="51" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="70" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="52" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="59" t="s">
+        <v>95</v>
+      </c>
+      <c r="H8" s="54" t="s">
         <v>78</v>
       </c>
-      <c r="I7" s="18"/>
-      <c r="J7" s="21"/>
-    </row>
-    <row r="8" spans="1:29" s="7" customFormat="1" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="118"/>
-      <c r="B8" s="65" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="65" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="84" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="F8" s="66" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" s="73" t="s">
-        <v>96</v>
-      </c>
-      <c r="H8" s="68" t="s">
-        <v>78</v>
-      </c>
-      <c r="I8" s="69"/>
-      <c r="J8" s="21"/>
+      <c r="I8" s="55"/>
+      <c r="J8" s="20"/>
       <c r="K8"/>
       <c r="L8"/>
       <c r="M8"/>
@@ -2116,496 +2148,480 @@
       <c r="AC8"/>
     </row>
     <row r="9" spans="1:29" ht="40.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="78" t="s">
+      <c r="A9" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="37" t="s">
+      <c r="B9" s="31" t="s">
         <v>79</v>
       </c>
-      <c r="C9" s="38" t="s">
+      <c r="C9" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="D9" s="39" t="s">
+      <c r="D9" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="40" t="s">
+      <c r="E9" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="F9" s="40" t="s">
+      <c r="F9" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="57" t="s">
+      <c r="G9" s="43" t="s">
+        <v>95</v>
+      </c>
+      <c r="H9" s="105" t="s">
+        <v>114</v>
+      </c>
+      <c r="I9" s="106" t="s">
+        <v>138</v>
+      </c>
+      <c r="J9" s="20"/>
+    </row>
+    <row r="10" spans="1:29" ht="42" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="80" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="44" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="66" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="45" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" s="45" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="56" t="s">
+        <v>97</v>
+      </c>
+      <c r="H10" s="72" t="s">
+        <v>114</v>
+      </c>
+      <c r="I10" s="49" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="121"/>
+      <c r="B11" s="32" t="s">
+        <v>144</v>
+      </c>
+      <c r="C11" s="32" t="s">
+        <v>145</v>
+      </c>
+      <c r="D11" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="34" t="s">
+        <v>59</v>
+      </c>
+      <c r="G11" s="122" t="s">
+        <v>97</v>
+      </c>
+      <c r="H11" s="42" t="s">
+        <v>78</v>
+      </c>
+      <c r="I11" s="123"/>
+    </row>
+    <row r="12" spans="1:29" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="78"/>
+      <c r="B12" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="51" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="52" t="s">
+        <v>98</v>
+      </c>
+      <c r="F12" s="51" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" s="71" t="s">
+        <v>97</v>
+      </c>
+      <c r="H12" s="54" t="s">
+        <v>78</v>
+      </c>
+      <c r="I12" s="55"/>
+    </row>
+    <row r="13" spans="1:29" ht="51.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="79" t="s">
+        <v>113</v>
+      </c>
+      <c r="B13" s="44" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="44" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" s="56" t="s">
+        <v>97</v>
+      </c>
+      <c r="H13" s="72" t="s">
+        <v>114</v>
+      </c>
+      <c r="I13" s="49" t="s">
+        <v>130</v>
+      </c>
+      <c r="J13" s="20"/>
+    </row>
+    <row r="14" spans="1:29" ht="51" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="77"/>
+      <c r="B14" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" s="57" t="s">
+        <v>97</v>
+      </c>
+      <c r="H14" s="72" t="s">
+        <v>114</v>
+      </c>
+      <c r="I14" s="19" t="s">
+        <v>131</v>
+      </c>
+      <c r="J14" s="20"/>
+    </row>
+    <row r="15" spans="1:29" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="78"/>
+      <c r="B15" s="51" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15" s="51" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" s="58" t="s">
+        <v>59</v>
+      </c>
+      <c r="G15" s="62" t="s">
         <v>96</v>
       </c>
-      <c r="H9" s="56" t="s">
+      <c r="H15" s="54" t="s">
         <v>78</v>
       </c>
-      <c r="I9" s="41"/>
-      <c r="J9" s="21"/>
-    </row>
-    <row r="10" spans="1:29" ht="42" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="101" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="58" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="58" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="80" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="59" t="s">
-        <v>60</v>
-      </c>
-      <c r="F10" s="59" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" s="70" t="s">
-        <v>98</v>
-      </c>
-      <c r="H10" s="62" t="s">
-        <v>78</v>
-      </c>
-      <c r="I10" s="63"/>
-    </row>
-    <row r="11" spans="1:29" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="99"/>
-      <c r="B11" s="65" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="65" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="65" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="66" t="s">
-        <v>99</v>
-      </c>
-      <c r="F11" s="65" t="s">
-        <v>20</v>
-      </c>
-      <c r="G11" s="85" t="s">
-        <v>98</v>
-      </c>
-      <c r="H11" s="68" t="s">
-        <v>78</v>
-      </c>
-      <c r="I11" s="69"/>
-    </row>
-    <row r="12" spans="1:29" ht="51.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="100" t="s">
-        <v>114</v>
-      </c>
-      <c r="B12" s="58" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="58" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="58" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="59" t="s">
-        <v>33</v>
-      </c>
-      <c r="F12" s="60" t="s">
-        <v>20</v>
-      </c>
-      <c r="G12" s="70" t="s">
-        <v>98</v>
-      </c>
-      <c r="H12" s="62" t="s">
-        <v>78</v>
-      </c>
-      <c r="I12" s="63" t="s">
-        <v>82</v>
-      </c>
-      <c r="J12" s="21"/>
-    </row>
-    <row r="13" spans="1:29" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="98"/>
-      <c r="B13" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="43" t="s">
-        <v>33</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="G13" s="71" t="s">
-        <v>98</v>
-      </c>
-      <c r="H13" s="64" t="s">
-        <v>78</v>
-      </c>
-      <c r="I13" s="20"/>
-      <c r="J13" s="21"/>
-    </row>
-    <row r="14" spans="1:29" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="99"/>
-      <c r="B14" s="65" t="s">
-        <v>93</v>
-      </c>
-      <c r="C14" s="65" t="s">
-        <v>94</v>
-      </c>
-      <c r="D14" s="65" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="66" t="s">
-        <v>20</v>
-      </c>
-      <c r="F14" s="72" t="s">
-        <v>59</v>
-      </c>
-      <c r="G14" s="76" t="s">
-        <v>97</v>
-      </c>
-      <c r="H14" s="68" t="s">
-        <v>78</v>
-      </c>
-      <c r="I14" s="69"/>
-      <c r="J14" s="21"/>
-    </row>
-    <row r="15" spans="1:29" ht="47.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="119" t="s">
+      <c r="I15" s="55"/>
+      <c r="J15" s="20"/>
+    </row>
+    <row r="16" spans="1:29" ht="47.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="98" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B16" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C16" s="11" t="s">
         <v>76</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="122" t="s">
-        <v>60</v>
-      </c>
-      <c r="F15" s="43" t="s">
-        <v>59</v>
-      </c>
-      <c r="G15" s="70" t="s">
-        <v>98</v>
-      </c>
-      <c r="H15" s="52" t="s">
-        <v>78</v>
-      </c>
-      <c r="I15" s="20"/>
-      <c r="J15" s="21"/>
-    </row>
-    <row r="16" spans="1:29" ht="48.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="119"/>
-      <c r="B16" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>74</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="122" t="s">
+      <c r="E16" s="74" t="s">
         <v>60</v>
       </c>
-      <c r="F16" s="43" t="s">
+      <c r="F16" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="G16" s="70" t="s">
-        <v>98</v>
-      </c>
-      <c r="H16" s="52" t="s">
+      <c r="G16" s="56" t="s">
+        <v>97</v>
+      </c>
+      <c r="H16" s="40" t="s">
         <v>78</v>
       </c>
-      <c r="I16" s="20"/>
-      <c r="J16" s="21"/>
-    </row>
-    <row r="17" spans="1:29" s="7" customFormat="1" ht="51.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="120"/>
-      <c r="B17" s="14" t="s">
+      <c r="I16" s="19"/>
+      <c r="J16" s="20"/>
+    </row>
+    <row r="17" spans="1:29" ht="48.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="98"/>
+      <c r="B17" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" s="74" t="s">
+        <v>60</v>
+      </c>
+      <c r="F17" s="36" t="s">
+        <v>59</v>
+      </c>
+      <c r="G17" s="56" t="s">
+        <v>97</v>
+      </c>
+      <c r="H17" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="I17" s="19"/>
+      <c r="J17" s="20"/>
+    </row>
+    <row r="18" spans="1:29" s="7" customFormat="1" ht="51.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="99"/>
+      <c r="B18" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C18" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D18" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="123" t="s">
+      <c r="E18" s="75" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="123" t="s">
+      <c r="F18" s="75" t="s">
         <v>59</v>
       </c>
-      <c r="G17" s="70" t="s">
-        <v>98</v>
-      </c>
-      <c r="H17" s="53" t="s">
+      <c r="G18" s="56" t="s">
+        <v>97</v>
+      </c>
+      <c r="H18" s="41" t="s">
         <v>78</v>
       </c>
-      <c r="I17" s="19"/>
-      <c r="J17" s="21"/>
-      <c r="K17"/>
-      <c r="L17"/>
-      <c r="M17"/>
-      <c r="N17"/>
-      <c r="O17"/>
-      <c r="P17"/>
-      <c r="Q17"/>
-      <c r="R17"/>
-      <c r="S17"/>
-      <c r="T17"/>
-      <c r="U17"/>
-      <c r="V17"/>
-      <c r="W17"/>
-      <c r="X17"/>
-      <c r="Y17"/>
-      <c r="Z17"/>
-      <c r="AA17"/>
-      <c r="AB17"/>
-      <c r="AC17"/>
-    </row>
-    <row r="18" spans="1:29" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="121" t="s">
+      <c r="I18" s="18"/>
+      <c r="J18" s="20"/>
+      <c r="K18"/>
+      <c r="L18"/>
+      <c r="M18"/>
+      <c r="N18"/>
+      <c r="O18"/>
+      <c r="P18"/>
+      <c r="Q18"/>
+      <c r="R18"/>
+      <c r="S18"/>
+      <c r="T18"/>
+      <c r="U18"/>
+      <c r="V18"/>
+      <c r="W18"/>
+      <c r="X18"/>
+      <c r="Y18"/>
+      <c r="Z18"/>
+      <c r="AA18"/>
+      <c r="AB18"/>
+      <c r="AC18"/>
+    </row>
+    <row r="19" spans="1:29" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="100" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="58" t="s">
+      <c r="B19" s="44" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="58" t="s">
+      <c r="C19" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="D18" s="58" t="s">
+      <c r="D19" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="59" t="s">
+      <c r="E19" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="F18" s="59" t="s">
+      <c r="F19" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="G18" s="74" t="s">
-        <v>97</v>
-      </c>
-      <c r="H18" s="62" t="s">
-        <v>78</v>
-      </c>
-      <c r="I18" s="63"/>
-      <c r="J18" s="21"/>
-    </row>
-    <row r="19" spans="1:29" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="98"/>
-      <c r="B19" s="11" t="s">
+      <c r="G19" s="60" t="s">
+        <v>96</v>
+      </c>
+      <c r="H19" s="72" t="s">
+        <v>114</v>
+      </c>
+      <c r="I19" s="49"/>
+      <c r="J19" s="20"/>
+    </row>
+    <row r="20" spans="1:29" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="77"/>
+      <c r="B20" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C20" s="11" t="s">
         <v>77</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E19" s="43" t="s">
-        <v>33</v>
-      </c>
-      <c r="F19" s="43" t="s">
-        <v>20</v>
-      </c>
-      <c r="G19" s="75" t="s">
-        <v>97</v>
-      </c>
-      <c r="H19" s="64" t="s">
-        <v>78</v>
-      </c>
-      <c r="I19" s="29"/>
-      <c r="J19" s="21"/>
-    </row>
-    <row r="20" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="98"/>
-      <c r="B20" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>47</v>
       </c>
       <c r="D20" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="43" t="s">
+      <c r="E20" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="F20" s="43" t="s">
+      <c r="F20" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G20" s="75" t="s">
-        <v>97</v>
-      </c>
-      <c r="H20" s="64" t="s">
-        <v>78</v>
-      </c>
-      <c r="I20" s="20"/>
-      <c r="J20" s="21"/>
-    </row>
-    <row r="21" spans="1:29" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="98"/>
+      <c r="G20" s="61" t="s">
+        <v>96</v>
+      </c>
+      <c r="H20" s="107" t="s">
+        <v>114</v>
+      </c>
+      <c r="I20" s="28"/>
+      <c r="J20" s="20"/>
+    </row>
+    <row r="21" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="77"/>
       <c r="B21" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E21" s="43" t="s">
+      <c r="E21" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="F21" s="43" t="s">
+      <c r="F21" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G21" s="75" t="s">
-        <v>97</v>
-      </c>
-      <c r="H21" s="64" t="s">
-        <v>78</v>
-      </c>
-      <c r="I21" s="20"/>
-      <c r="J21" s="21"/>
-    </row>
-    <row r="22" spans="1:29" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="98"/>
+      <c r="G21" s="61" t="s">
+        <v>96</v>
+      </c>
+      <c r="H21" s="107" t="s">
+        <v>114</v>
+      </c>
+      <c r="I21" s="19"/>
+      <c r="J21" s="20"/>
+    </row>
+    <row r="22" spans="1:29" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="77"/>
       <c r="B22" s="11" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D22" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E22" s="43" t="s">
+      <c r="E22" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="F22" s="43" t="s">
+      <c r="F22" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G22" s="75" t="s">
-        <v>97</v>
-      </c>
-      <c r="H22" s="64" t="s">
-        <v>78</v>
-      </c>
-      <c r="I22" s="20"/>
-      <c r="J22" s="21"/>
-    </row>
-    <row r="23" spans="1:29" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="98"/>
+      <c r="G22" s="61" t="s">
+        <v>96</v>
+      </c>
+      <c r="H22" s="107" t="s">
+        <v>114</v>
+      </c>
+      <c r="I22" s="19"/>
+      <c r="J22" s="20"/>
+    </row>
+    <row r="23" spans="1:29" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="77"/>
       <c r="B23" s="11" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D23" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E23" s="43" t="s">
+      <c r="E23" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="F23" s="43" t="s">
+      <c r="F23" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G23" s="75" t="s">
-        <v>97</v>
-      </c>
-      <c r="H23" s="64" t="s">
+      <c r="G23" s="61" t="s">
+        <v>96</v>
+      </c>
+      <c r="H23" s="50" t="s">
         <v>78</v>
       </c>
-      <c r="I23" s="28"/>
-      <c r="J23" s="21"/>
-    </row>
-    <row r="24" spans="1:29" s="7" customFormat="1" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="99"/>
-      <c r="B24" s="65" t="s">
+      <c r="I23" s="19"/>
+      <c r="J23" s="20"/>
+    </row>
+    <row r="24" spans="1:29" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="77"/>
+      <c r="B24" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E24" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="F24" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="G24" s="61" t="s">
+        <v>96</v>
+      </c>
+      <c r="H24" s="107" t="s">
+        <v>114</v>
+      </c>
+      <c r="I24" s="27"/>
+      <c r="J24" s="20"/>
+    </row>
+    <row r="25" spans="1:29" s="7" customFormat="1" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="78"/>
+      <c r="B25" s="51" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="65" t="s">
+      <c r="C25" s="51" t="s">
         <v>53</v>
       </c>
-      <c r="D24" s="65" t="s">
+      <c r="D25" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="66" t="s">
+      <c r="E25" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="F24" s="66" t="s">
+      <c r="F25" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="G24" s="76" t="s">
-        <v>97</v>
-      </c>
-      <c r="H24" s="68" t="s">
-        <v>78</v>
-      </c>
-      <c r="I24" s="69"/>
-      <c r="J24" s="21"/>
-      <c r="K24"/>
-      <c r="L24"/>
-      <c r="M24"/>
-      <c r="N24"/>
-      <c r="O24"/>
-      <c r="P24"/>
-      <c r="Q24"/>
-      <c r="R24"/>
-      <c r="S24"/>
-      <c r="T24"/>
-      <c r="U24"/>
-      <c r="V24"/>
-      <c r="W24"/>
-      <c r="X24"/>
-      <c r="Y24"/>
-      <c r="Z24"/>
-      <c r="AA24"/>
-      <c r="AB24"/>
-      <c r="AC24"/>
-    </row>
-    <row r="25" spans="1:29" s="15" customFormat="1" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="113" t="s">
-        <v>54</v>
-      </c>
-      <c r="B25" s="58" t="s">
-        <v>56</v>
-      </c>
-      <c r="C25" s="58" t="s">
-        <v>61</v>
-      </c>
-      <c r="D25" s="58" t="s">
-        <v>19</v>
-      </c>
-      <c r="E25" s="59" t="s">
-        <v>33</v>
-      </c>
-      <c r="F25" s="59" t="s">
-        <v>59</v>
-      </c>
-      <c r="G25" s="70" t="s">
-        <v>98</v>
-      </c>
-      <c r="H25" s="62" t="s">
-        <v>78</v>
-      </c>
-      <c r="I25" s="63"/>
-      <c r="J25"/>
+      <c r="G25" s="62" t="s">
+        <v>96</v>
+      </c>
+      <c r="H25" s="108" t="s">
+        <v>114</v>
+      </c>
+      <c r="I25" s="55"/>
+      <c r="J25" s="20"/>
       <c r="K25"/>
       <c r="L25"/>
       <c r="M25"/>
@@ -2626,132 +2642,158 @@
       <c r="AB25"/>
       <c r="AC25"/>
     </row>
-    <row r="26" spans="1:29" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="114"/>
-      <c r="B26" s="11" t="s">
+    <row r="26" spans="1:29" s="15" customFormat="1" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="92" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="44" t="s">
+        <v>61</v>
+      </c>
+      <c r="D26" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="F26" s="45" t="s">
+        <v>59</v>
+      </c>
+      <c r="G26" s="56" t="s">
+        <v>97</v>
+      </c>
+      <c r="H26" s="48" t="s">
+        <v>78</v>
+      </c>
+      <c r="I26" s="49"/>
+      <c r="J26"/>
+      <c r="K26"/>
+      <c r="L26"/>
+      <c r="M26"/>
+      <c r="N26"/>
+      <c r="O26"/>
+      <c r="P26"/>
+      <c r="Q26"/>
+      <c r="R26"/>
+      <c r="S26"/>
+      <c r="T26"/>
+      <c r="U26"/>
+      <c r="V26"/>
+      <c r="W26"/>
+      <c r="X26"/>
+      <c r="Y26"/>
+      <c r="Z26"/>
+      <c r="AA26"/>
+      <c r="AB26"/>
+      <c r="AC26"/>
+    </row>
+    <row r="27" spans="1:29" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="93"/>
+      <c r="B27" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="C27" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="C26" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="D26" s="11" t="s">
+      <c r="D27" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E27" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="F27" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="G27" s="57" t="s">
+        <v>97</v>
+      </c>
+      <c r="H27" s="50" t="s">
+        <v>78</v>
+      </c>
+      <c r="I27" s="19"/>
+    </row>
+    <row r="28" spans="1:29" s="17" customFormat="1" ht="55.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="94"/>
+      <c r="B28" s="51" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="51" t="s">
+        <v>62</v>
+      </c>
+      <c r="D28" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="E28" s="52" t="s">
+        <v>33</v>
+      </c>
+      <c r="F28" s="58" t="s">
         <v>20</v>
       </c>
-      <c r="G26" s="71" t="s">
-        <v>98</v>
-      </c>
-      <c r="H26" s="64" t="s">
-        <v>78</v>
-      </c>
-      <c r="I26" s="20"/>
-    </row>
-    <row r="27" spans="1:29" s="17" customFormat="1" ht="55.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="115"/>
-      <c r="B27" s="65" t="s">
-        <v>57</v>
-      </c>
-      <c r="C27" s="65" t="s">
-        <v>62</v>
-      </c>
-      <c r="D27" s="65" t="s">
+      <c r="G28" s="59" t="s">
+        <v>95</v>
+      </c>
+      <c r="H28" s="108" t="s">
+        <v>114</v>
+      </c>
+      <c r="I28" s="55" t="s">
+        <v>132</v>
+      </c>
+      <c r="J28"/>
+      <c r="K28"/>
+      <c r="L28"/>
+      <c r="M28"/>
+      <c r="N28"/>
+      <c r="O28"/>
+      <c r="P28"/>
+      <c r="Q28"/>
+      <c r="R28"/>
+      <c r="S28"/>
+      <c r="T28"/>
+      <c r="U28"/>
+      <c r="V28"/>
+      <c r="W28"/>
+      <c r="X28"/>
+      <c r="Y28"/>
+      <c r="Z28"/>
+      <c r="AA28"/>
+      <c r="AB28"/>
+      <c r="AC28"/>
+    </row>
+    <row r="29" spans="1:29" ht="28.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="76" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29" s="44" t="s">
+        <v>99</v>
+      </c>
+      <c r="C29" s="44" t="s">
+        <v>104</v>
+      </c>
+      <c r="D29" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="E27" s="66" t="s">
+      <c r="E29" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="F27" s="72" t="s">
+      <c r="F29" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G27" s="73" t="s">
-        <v>96</v>
-      </c>
-      <c r="H27" s="68" t="s">
-        <v>78</v>
-      </c>
-      <c r="I27" s="69"/>
-      <c r="J27"/>
-      <c r="K27"/>
-      <c r="L27"/>
-      <c r="M27"/>
-      <c r="N27"/>
-      <c r="O27"/>
-      <c r="P27"/>
-      <c r="Q27"/>
-      <c r="R27"/>
-      <c r="S27"/>
-      <c r="T27"/>
-      <c r="U27"/>
-      <c r="V27"/>
-      <c r="W27"/>
-      <c r="X27"/>
-      <c r="Y27"/>
-      <c r="Z27"/>
-      <c r="AA27"/>
-      <c r="AB27"/>
-      <c r="AC27"/>
-    </row>
-    <row r="28" spans="1:29" ht="28.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="97" t="s">
-        <v>35</v>
-      </c>
-      <c r="B28" s="58" t="s">
+      <c r="G29" s="47" t="s">
+        <v>94</v>
+      </c>
+      <c r="H29" s="72" t="s">
+        <v>114</v>
+      </c>
+      <c r="I29" s="49" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="30" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="77"/>
+      <c r="B30" s="11" t="s">
         <v>100</v>
-      </c>
-      <c r="C28" s="58" t="s">
-        <v>105</v>
-      </c>
-      <c r="D28" s="58" t="s">
-        <v>19</v>
-      </c>
-      <c r="E28" s="59" t="s">
-        <v>33</v>
-      </c>
-      <c r="F28" s="60" t="s">
-        <v>20</v>
-      </c>
-      <c r="G28" s="61" t="s">
-        <v>95</v>
-      </c>
-      <c r="H28" s="62" t="s">
-        <v>78</v>
-      </c>
-      <c r="I28" s="63"/>
-    </row>
-    <row r="29" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="98"/>
-      <c r="B29" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="D29" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E29" s="43" t="s">
-        <v>33</v>
-      </c>
-      <c r="F29" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="G29" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="H29" s="64" t="s">
-        <v>78</v>
-      </c>
-      <c r="I29" s="20"/>
-    </row>
-    <row r="30" spans="1:29" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="98"/>
-      <c r="B30" s="11" t="s">
-        <v>102</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>103</v>
@@ -2759,114 +2801,94 @@
       <c r="D30" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E30" s="10" t="s">
-        <v>20</v>
+      <c r="E30" s="36" t="s">
+        <v>33</v>
       </c>
       <c r="F30" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="G30" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="H30" s="64" t="s">
+      <c r="G30" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="H30" s="50" t="s">
         <v>78</v>
       </c>
-      <c r="I30" s="20"/>
-    </row>
-    <row r="31" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="98"/>
+      <c r="I30" s="19"/>
+    </row>
+    <row r="31" spans="1:29" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="77"/>
       <c r="B31" s="11" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E31" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="F31" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="G31" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="H31" s="64" t="s">
+      <c r="E31" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F31" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="G31" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="H31" s="50" t="s">
         <v>78</v>
       </c>
-      <c r="I31" s="20"/>
-    </row>
-    <row r="32" spans="1:29" s="16" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="98"/>
+      <c r="I31" s="19"/>
+    </row>
+    <row r="32" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="77"/>
       <c r="B32" s="11" t="s">
-        <v>55</v>
+        <v>105</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="D32" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E32" s="43" t="s">
-        <v>33</v>
-      </c>
-      <c r="F32" s="43" t="s">
-        <v>20</v>
-      </c>
-      <c r="G32" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="H32" s="64" t="s">
+      <c r="E32" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="G32" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="H32" s="50" t="s">
         <v>78</v>
       </c>
-      <c r="I32" s="20"/>
-      <c r="J32"/>
-      <c r="K32"/>
-      <c r="L32"/>
-      <c r="M32"/>
-      <c r="N32"/>
-      <c r="O32"/>
-      <c r="P32"/>
-      <c r="Q32"/>
-      <c r="R32"/>
-      <c r="S32"/>
-      <c r="T32"/>
-      <c r="U32"/>
-      <c r="V32"/>
-      <c r="W32"/>
-      <c r="X32"/>
-      <c r="Y32"/>
-      <c r="Z32"/>
-      <c r="AA32"/>
-      <c r="AB32"/>
-      <c r="AC32"/>
-    </row>
-    <row r="33" spans="1:29" s="16" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="98"/>
+      <c r="I32" s="19"/>
+    </row>
+    <row r="33" spans="1:29" s="16" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="77"/>
       <c r="B33" s="11" t="s">
-        <v>108</v>
+        <v>55</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="D33" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E33" s="43" t="s">
+      <c r="E33" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="F33" s="43" t="s">
+      <c r="F33" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G33" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="H33" s="64" t="s">
+      <c r="G33" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="H33" s="50" t="s">
         <v>78</v>
       </c>
-      <c r="I33" s="20"/>
+      <c r="I33" s="19"/>
       <c r="J33"/>
       <c r="K33"/>
       <c r="L33"/>
@@ -2888,30 +2910,30 @@
       <c r="AB33"/>
       <c r="AC33"/>
     </row>
-    <row r="34" spans="1:29" s="16" customFormat="1" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="99"/>
-      <c r="B34" s="65" t="s">
-        <v>110</v>
-      </c>
-      <c r="C34" s="65" t="s">
-        <v>111</v>
-      </c>
-      <c r="D34" s="65" t="s">
+    <row r="34" spans="1:29" s="16" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="77"/>
+      <c r="B34" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="D34" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E34" s="66" t="s">
-        <v>33</v>
-      </c>
-      <c r="F34" s="66" t="s">
+      <c r="E34" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G34" s="67" t="s">
-        <v>95</v>
-      </c>
-      <c r="H34" s="68" t="s">
+      <c r="F34" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="G34" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="H34" s="50" t="s">
         <v>78</v>
       </c>
-      <c r="I34" s="69"/>
+      <c r="I34" s="19"/>
       <c r="J34"/>
       <c r="K34"/>
       <c r="L34"/>
@@ -2933,21 +2955,158 @@
       <c r="AB34"/>
       <c r="AC34"/>
     </row>
-    <row r="35" spans="1:29" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="1:29" s="16" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="77"/>
+      <c r="B35" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E35" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="F35" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="G35" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="H35" s="107" t="s">
+        <v>114</v>
+      </c>
+      <c r="I35" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="J35"/>
+      <c r="K35"/>
+      <c r="L35"/>
+      <c r="M35"/>
+      <c r="N35"/>
+      <c r="O35"/>
+      <c r="P35"/>
+      <c r="Q35"/>
+      <c r="R35"/>
+      <c r="S35"/>
+      <c r="T35"/>
+      <c r="U35"/>
+      <c r="V35"/>
+      <c r="W35"/>
+      <c r="X35"/>
+      <c r="Y35"/>
+      <c r="Z35"/>
+      <c r="AA35"/>
+      <c r="AB35"/>
+      <c r="AC35"/>
+    </row>
+    <row r="36" spans="1:29" s="16" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="77"/>
+      <c r="B36" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="C36" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="D36" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E36" s="36" t="s">
+        <v>33</v>
+      </c>
+      <c r="F36" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="G36" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="H36" s="50" t="s">
+        <v>78</v>
+      </c>
+      <c r="I36" s="19"/>
+      <c r="J36"/>
+      <c r="K36"/>
+      <c r="L36"/>
+      <c r="M36"/>
+      <c r="N36"/>
+      <c r="O36"/>
+      <c r="P36"/>
+      <c r="Q36"/>
+      <c r="R36"/>
+      <c r="S36"/>
+      <c r="T36"/>
+      <c r="U36"/>
+      <c r="V36"/>
+      <c r="W36"/>
+      <c r="X36"/>
+      <c r="Y36"/>
+      <c r="Z36"/>
+      <c r="AA36"/>
+      <c r="AB36"/>
+      <c r="AC36"/>
+    </row>
+    <row r="37" spans="1:29" s="16" customFormat="1" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="78"/>
+      <c r="B37" s="51" t="s">
+        <v>109</v>
+      </c>
+      <c r="C37" s="51" t="s">
+        <v>110</v>
+      </c>
+      <c r="D37" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37" s="52" t="s">
+        <v>33</v>
+      </c>
+      <c r="F37" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="G37" s="53" t="s">
+        <v>94</v>
+      </c>
+      <c r="H37" s="54" t="s">
+        <v>78</v>
+      </c>
+      <c r="I37" s="55"/>
+      <c r="J37"/>
+      <c r="K37"/>
+      <c r="L37"/>
+      <c r="M37"/>
+      <c r="N37"/>
+      <c r="O37"/>
+      <c r="P37"/>
+      <c r="Q37"/>
+      <c r="R37"/>
+      <c r="S37"/>
+      <c r="T37"/>
+      <c r="U37"/>
+      <c r="V37"/>
+      <c r="W37"/>
+      <c r="X37"/>
+      <c r="Y37"/>
+      <c r="Z37"/>
+      <c r="AA37"/>
+      <c r="AB37"/>
+      <c r="AC37"/>
+    </row>
+    <row r="38" spans="1:29" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="G5:G34" xr:uid="{4AB4A1F4-D2AB-4474-B05F-C8B13F4E557C}"/>
+  <autoFilter ref="H5:H37" xr:uid="{4AB4A1F4-D2AB-4474-B05F-C8B13F4E557C}"/>
   <mergeCells count="11">
-    <mergeCell ref="A28:A34"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A29:A37"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="A10:A12"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="B4:I4"/>
-    <mergeCell ref="A25:A27"/>
+    <mergeCell ref="A26:A28"/>
     <mergeCell ref="A6:A8"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="A18:A24"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="A19:A25"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B4" r:id="rId1" xr:uid="{73359DB6-C291-4AB2-82A3-BE2171E1A73F}"/>
@@ -2959,7 +3118,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{748CED0D-D7CE-4618-A56E-B7666AE2995E}">
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.42578125" style="1" customWidth="1"/>
@@ -2972,320 +3131,367 @@
     <col min="8" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="37.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="88" t="s">
+    <row r="1" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="101" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="89"/>
-      <c r="D1" s="89"/>
-      <c r="E1" s="89"/>
-      <c r="F1" s="90"/>
-    </row>
-    <row r="2" spans="1:7" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="46" t="s">
-        <v>84</v>
-      </c>
-      <c r="B2" s="91" t="s">
+      <c r="B1" s="102"/>
+      <c r="C1" s="102"/>
+      <c r="D1" s="102"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="111"/>
+    </row>
+    <row r="2" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="39" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="103" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2" s="104"/>
+      <c r="D2" s="104"/>
+      <c r="E2" s="104"/>
+      <c r="F2" s="104"/>
+      <c r="G2" s="112"/>
+    </row>
+    <row r="3" spans="1:8" s="26" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="109" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="113" t="s">
+        <v>88</v>
+      </c>
+      <c r="H3" s="110"/>
+    </row>
+    <row r="4" spans="1:8" ht="225.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="114" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="114" t="s">
         <v>87</v>
       </c>
-      <c r="C2" s="92"/>
-      <c r="D2" s="92"/>
-      <c r="E2" s="92"/>
-      <c r="F2" s="93"/>
-    </row>
-    <row r="3" spans="1:7" s="27" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="24" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="25" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="225.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C4" s="54" t="s">
+      <c r="C4" s="115" t="s">
+        <v>124</v>
+      </c>
+      <c r="D4" s="114" t="s">
         <v>125</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="114" t="s">
         <v>126</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="114" t="s">
         <v>127</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="G4" s="114" t="s">
         <v>128</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="143.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="22" t="s">
+    </row>
+    <row r="5" spans="1:8" ht="143.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="114" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="114" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="54" t="s">
-        <v>86</v>
-      </c>
-      <c r="F5" s="23"/>
-    </row>
-    <row r="6" spans="1:7" ht="191.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
+      <c r="C5" s="115" t="s">
+        <v>85</v>
+      </c>
+      <c r="D5" s="114" t="s">
+        <v>133</v>
+      </c>
+      <c r="E5" s="114" t="s">
+        <v>134</v>
+      </c>
+      <c r="F5" s="114" t="s">
+        <v>135</v>
+      </c>
+      <c r="G5" s="114" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="191.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="114" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="114" t="s">
         <v>66</v>
       </c>
-      <c r="C6" s="54" t="s">
-        <v>86</v>
-      </c>
-      <c r="F6" s="23"/>
-    </row>
-    <row r="7" spans="1:7" ht="115.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="22" t="s">
+      <c r="C6" s="115" t="s">
+        <v>85</v>
+      </c>
+      <c r="D6" s="114"/>
+      <c r="E6" s="114"/>
+      <c r="F6" s="114"/>
+      <c r="G6" s="114"/>
+    </row>
+    <row r="7" spans="1:8" ht="115.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="114" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="114" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="55" t="s">
-        <v>86</v>
-      </c>
-      <c r="F7" s="23"/>
-    </row>
-    <row r="8" spans="1:7" s="31" customFormat="1" ht="227.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="30" t="s">
+      <c r="C7" s="115" t="s">
+        <v>85</v>
+      </c>
+      <c r="D7" s="114"/>
+      <c r="E7" s="114"/>
+      <c r="F7" s="114"/>
+      <c r="G7" s="114"/>
+    </row>
+    <row r="8" spans="1:8" s="29" customFormat="1" ht="227.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="116" t="s">
         <v>72</v>
       </c>
-      <c r="B8" s="94" t="s">
+      <c r="B8" s="117" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="54" t="s">
-        <v>86</v>
-      </c>
-      <c r="E8" s="49"/>
-      <c r="F8" s="32"/>
-    </row>
-    <row r="9" spans="1:7" ht="238.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="33" t="s">
+      <c r="C8" s="115" t="s">
+        <v>85</v>
+      </c>
+      <c r="D8" s="114"/>
+      <c r="E8" s="118"/>
+      <c r="F8" s="114"/>
+      <c r="G8" s="114"/>
+    </row>
+    <row r="9" spans="1:8" ht="238.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="114" t="s">
         <v>68</v>
       </c>
-      <c r="B9" s="95"/>
-      <c r="C9" s="54" t="s">
-        <v>86</v>
-      </c>
-      <c r="E9" s="50"/>
-      <c r="F9" s="23"/>
-    </row>
-    <row r="10" spans="1:7" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="47" t="s">
+      <c r="B9" s="117"/>
+      <c r="C9" s="115" t="s">
+        <v>85</v>
+      </c>
+      <c r="D9" s="114"/>
+      <c r="E9" s="118"/>
+      <c r="F9" s="114"/>
+      <c r="G9" s="114"/>
+    </row>
+    <row r="10" spans="1:8" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="119" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="95"/>
-      <c r="C10" s="48" t="s">
-        <v>86</v>
-      </c>
-      <c r="D10" s="48"/>
-      <c r="E10" s="50"/>
-      <c r="F10" s="23"/>
-    </row>
-    <row r="11" spans="1:7" ht="145.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="33" t="s">
+      <c r="B10" s="117"/>
+      <c r="C10" s="119" t="s">
+        <v>85</v>
+      </c>
+      <c r="D10" s="119"/>
+      <c r="E10" s="118"/>
+      <c r="F10" s="114"/>
+      <c r="G10" s="114"/>
+    </row>
+    <row r="11" spans="1:8" ht="145.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="114" t="s">
         <v>70</v>
       </c>
-      <c r="B11" s="95"/>
-      <c r="C11" s="54" t="s">
-        <v>86</v>
-      </c>
-      <c r="E11" s="50"/>
-      <c r="F11" s="23"/>
-    </row>
-    <row r="12" spans="1:7" s="35" customFormat="1" ht="102" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="34" t="s">
+      <c r="B11" s="117"/>
+      <c r="C11" s="115" t="s">
+        <v>85</v>
+      </c>
+      <c r="D11" s="114"/>
+      <c r="E11" s="118"/>
+      <c r="F11" s="114"/>
+      <c r="G11" s="114"/>
+    </row>
+    <row r="12" spans="1:8" s="30" customFormat="1" ht="102" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="114" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="96"/>
-      <c r="C12" s="55" t="s">
-        <v>86</v>
-      </c>
-      <c r="E12" s="51"/>
-      <c r="F12" s="36"/>
-    </row>
-    <row r="13" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="22" t="s">
+      <c r="B12" s="117"/>
+      <c r="C12" s="115" t="s">
+        <v>85</v>
+      </c>
+      <c r="D12" s="114"/>
+      <c r="E12" s="118"/>
+      <c r="F12" s="114"/>
+      <c r="G12" s="114"/>
+    </row>
+    <row r="13" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="114" t="s">
+        <v>116</v>
+      </c>
+      <c r="B13" s="114" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" s="115" t="s">
+        <v>85</v>
+      </c>
+      <c r="D13" s="114"/>
+      <c r="E13" s="114"/>
+      <c r="F13" s="114"/>
+      <c r="G13" s="114"/>
+    </row>
+    <row r="14" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="114" t="s">
         <v>117</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B14" s="114" t="s">
         <v>120</v>
       </c>
-      <c r="C13" s="54" t="s">
-        <v>86</v>
-      </c>
-      <c r="F13" s="23"/>
-    </row>
-    <row r="14" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="22" t="s">
+      <c r="C14" s="115" t="s">
+        <v>85</v>
+      </c>
+      <c r="D14" s="114"/>
+      <c r="E14" s="114"/>
+      <c r="F14" s="114"/>
+      <c r="G14" s="114"/>
+    </row>
+    <row r="15" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="114" t="s">
         <v>118</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B15" s="114" t="s">
         <v>121</v>
       </c>
-      <c r="C14" s="54" t="s">
-        <v>86</v>
-      </c>
-      <c r="F14" s="23"/>
-    </row>
-    <row r="15" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="22" t="s">
-        <v>119</v>
-      </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="115" t="s">
+        <v>85</v>
+      </c>
+      <c r="D15" s="114"/>
+      <c r="E15" s="114"/>
+      <c r="F15" s="114"/>
+      <c r="G15" s="114"/>
+    </row>
+    <row r="16" spans="1:8" ht="84" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="114" t="s">
         <v>122</v>
       </c>
-      <c r="C15" s="54" t="s">
-        <v>86</v>
-      </c>
-      <c r="F15" s="23"/>
-    </row>
-    <row r="16" spans="1:7" ht="84" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="22" t="s">
+      <c r="B16" s="114" t="s">
         <v>123</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="F16" s="23"/>
-    </row>
-    <row r="17" spans="1:6" ht="99.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="22"/>
-      <c r="F17" s="23"/>
-    </row>
-    <row r="18" spans="1:6" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="22"/>
-      <c r="F18" s="23"/>
-    </row>
-    <row r="19" spans="1:6" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="22"/>
-      <c r="F19" s="23"/>
-    </row>
-    <row r="20" spans="1:6" ht="78" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="22"/>
-      <c r="F20" s="23"/>
-    </row>
-    <row r="21" spans="1:6" ht="93" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="22"/>
-      <c r="F21" s="23"/>
-    </row>
-    <row r="22" spans="1:6" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="22"/>
-      <c r="F22" s="23"/>
-    </row>
-    <row r="23" spans="1:6" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="22"/>
-      <c r="F23" s="23"/>
-    </row>
-    <row r="24" spans="1:6" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="22"/>
-      <c r="F24" s="23"/>
-    </row>
-    <row r="25" spans="1:6" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="22"/>
-      <c r="F25" s="23"/>
-    </row>
-    <row r="26" spans="1:6" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="22"/>
-      <c r="F26" s="23"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="22"/>
-      <c r="F27" s="23"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="22"/>
-      <c r="F28" s="23"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="22"/>
-      <c r="F29" s="23"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="22"/>
-      <c r="F30" s="23"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="22"/>
-      <c r="F31" s="23"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="22"/>
-      <c r="F32" s="23"/>
+      <c r="C16" s="114"/>
+      <c r="D16" s="114"/>
+      <c r="E16" s="114"/>
+      <c r="F16" s="114"/>
+      <c r="G16" s="114"/>
+    </row>
+    <row r="17" spans="1:7" ht="99.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="114"/>
+      <c r="B17" s="114"/>
+      <c r="C17" s="114"/>
+      <c r="D17" s="114"/>
+      <c r="E17" s="114"/>
+      <c r="F17" s="114"/>
+      <c r="G17" s="114"/>
+    </row>
+    <row r="18" spans="1:7" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="21"/>
+      <c r="F18" s="22"/>
+    </row>
+    <row r="19" spans="1:7" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="21"/>
+      <c r="F19" s="22"/>
+    </row>
+    <row r="20" spans="1:7" ht="78" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="21"/>
+      <c r="F20" s="22"/>
+    </row>
+    <row r="21" spans="1:7" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="21"/>
+      <c r="F21" s="22"/>
+    </row>
+    <row r="22" spans="1:7" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="21"/>
+      <c r="F22" s="22"/>
+    </row>
+    <row r="23" spans="1:7" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="21"/>
+      <c r="F23" s="22"/>
+    </row>
+    <row r="24" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="21"/>
+      <c r="F24" s="22"/>
+    </row>
+    <row r="25" spans="1:7" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="21"/>
+      <c r="F25" s="22"/>
+    </row>
+    <row r="26" spans="1:7" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="21"/>
+      <c r="F26" s="22"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="21"/>
+      <c r="F27" s="22"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="21"/>
+      <c r="F28" s="22"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="21"/>
+      <c r="F29" s="22"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="21"/>
+      <c r="F30" s="22"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="21"/>
+      <c r="F31" s="22"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="21"/>
+      <c r="F32" s="22"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="22"/>
-      <c r="F33" s="23"/>
+      <c r="A33" s="21"/>
+      <c r="F33" s="22"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="22"/>
-      <c r="F34" s="23"/>
+      <c r="A34" s="21"/>
+      <c r="F34" s="22"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="22"/>
-      <c r="F35" s="23"/>
+      <c r="A35" s="21"/>
+      <c r="F35" s="22"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="22"/>
-      <c r="F36" s="23"/>
+      <c r="A36" s="21"/>
+      <c r="F36" s="22"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="22"/>
-      <c r="F37" s="23"/>
+      <c r="A37" s="21"/>
+      <c r="F37" s="22"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="22"/>
-      <c r="F38" s="23"/>
+      <c r="A38" s="21"/>
+      <c r="F38" s="22"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="22"/>
-      <c r="F39" s="23"/>
+      <c r="A39" s="21"/>
+      <c r="F39" s="22"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="22"/>
-      <c r="F40" s="23"/>
+      <c r="A40" s="21"/>
+      <c r="F40" s="22"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="22"/>
-      <c r="F41" s="23"/>
+      <c r="A41" s="21"/>
+      <c r="F41" s="22"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="22"/>
-      <c r="F42" s="23"/>
+      <c r="A42" s="21"/>
+      <c r="F42" s="22"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="22"/>
-      <c r="F43" s="23"/>
+      <c r="A43" s="21"/>
+      <c r="F43" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3558,15 +3764,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="ff8a4b2e-b0c8-4039-a689-d1a7f36f4382">
@@ -3576,6 +3773,15 @@
     <Notes xmlns="ff8a4b2e-b0c8-4039-a689-d1a7f36f4382" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3598,14 +3804,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8F3069D-89E7-4007-93BF-1DB2942FF756}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76F271AB-EFB2-4823-A2F0-9F2289E658DB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3616,4 +3814,12 @@
     <ds:schemaRef ds:uri="f716dd8a-49a0-4c40-b209-038e1651b548"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8F3069D-89E7-4007-93BF-1DB2942FF756}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
added Level2, tilemap, edited tileset
</commit_message>
<xml_diff>
--- a/Red Team Tracebility and Testing.xlsx
+++ b/Red Team Tracebility and Testing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Program Files\Epic Games\UE_5.7\redteam\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD5AE3FF-7369-4349-92CA-CA37A00F6F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8409E52F-DFBA-4DAB-AB3C-531532A5DFE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{19EF330C-6F54-4365-A47E-10806019DE9B}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Test Plan" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Traceability Matrix'!$H$5:$H$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Traceability Matrix'!$G$5:$G$37</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="148">
   <si>
     <t>Prototype Title:</t>
   </si>
@@ -521,9 +521,6 @@
     <t>Added player Health Pickups with a  temp heart model. -Nathen Reed</t>
   </si>
   <si>
-    <t>Checkpoints added with temp Placeholder. -Nathen Reed</t>
-  </si>
-  <si>
     <t>Big deathzone added that resets player to respawn point. -Nathen Reed</t>
   </si>
   <si>
@@ -567,6 +564,15 @@
   </si>
   <si>
     <t>Collectable coins they stay tracked on UI.</t>
+  </si>
+  <si>
+    <t>Final Release</t>
+  </si>
+  <si>
+    <t>Added collectible coins that are tracked between stages, and displayed with a widget. -Nathen Reed</t>
+  </si>
+  <si>
+    <t>Checkpoint Updated With custom FB. -Nathen Reed</t>
   </si>
 </sst>
 </file>
@@ -1261,7 +1267,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="124">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1366,7 +1372,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="13" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1454,95 +1459,8 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1572,25 +1490,109 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1912,7 +1914,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB4A1F4-D2AB-4474-B05F-C8B13F4E557C}">
-  <dimension ref="A1:AC38"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:AC37"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" style="1" customWidth="1"/>
@@ -1928,30 +1931,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="100" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
-      <c r="G1" s="85"/>
-      <c r="H1" s="85"/>
-      <c r="I1" s="85"/>
+      <c r="B1" s="101"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
+      <c r="E1" s="101"/>
+      <c r="F1" s="101"/>
+      <c r="G1" s="101"/>
+      <c r="H1" s="101"/>
+      <c r="I1" s="101"/>
     </row>
     <row r="2" spans="1:29" s="3" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="81"/>
-      <c r="C2" s="82"/>
-      <c r="D2" s="82"/>
-      <c r="E2" s="82"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="82"/>
-      <c r="H2" s="82"/>
-      <c r="I2" s="83"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
+      <c r="I2" s="99"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
@@ -1970,52 +1973,52 @@
       <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="86" t="s">
+      <c r="B3" s="102" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="87"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="87"/>
-      <c r="F3" s="87"/>
-      <c r="G3" s="87"/>
-      <c r="H3" s="87"/>
-      <c r="I3" s="88"/>
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="103"/>
+      <c r="G3" s="103"/>
+      <c r="H3" s="103"/>
+      <c r="I3" s="104"/>
     </row>
     <row r="4" spans="1:29" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="38" t="s">
         <v>83</v>
       </c>
-      <c r="B4" s="89" t="s">
+      <c r="B4" s="105" t="s">
         <v>86</v>
       </c>
-      <c r="C4" s="90"/>
-      <c r="D4" s="90"/>
-      <c r="E4" s="90"/>
-      <c r="F4" s="90"/>
-      <c r="G4" s="90"/>
-      <c r="H4" s="90"/>
-      <c r="I4" s="91"/>
+      <c r="C4" s="106"/>
+      <c r="D4" s="106"/>
+      <c r="E4" s="106"/>
+      <c r="F4" s="106"/>
+      <c r="G4" s="106"/>
+      <c r="H4" s="106"/>
+      <c r="I4" s="107"/>
     </row>
     <row r="5" spans="1:29" s="2" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="63" t="s">
+      <c r="A5" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="63" t="s">
+      <c r="B5" s="62" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="63" t="s">
+      <c r="C5" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="63" t="s">
+      <c r="D5" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="63" t="s">
+      <c r="E5" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="63" t="s">
+      <c r="F5" s="62" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="63" t="s">
+      <c r="G5" s="62" t="s">
         <v>15</v>
       </c>
       <c r="H5" s="35" t="s">
@@ -2025,32 +2028,32 @@
         <v>89</v>
       </c>
     </row>
-    <row r="6" spans="1:29" s="8" customFormat="1" ht="46.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="95" t="s">
+    <row r="6" spans="1:29" s="8" customFormat="1" ht="46.5" hidden="1" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="111" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="65" t="s">
+      <c r="B6" s="64" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="66" t="s">
+      <c r="C6" s="65" t="s">
         <v>81</v>
       </c>
-      <c r="D6" s="66" t="s">
+      <c r="D6" s="65" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="45" t="s">
+      <c r="E6" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="46" t="s">
+      <c r="F6" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="67" t="s">
+      <c r="G6" s="66" t="s">
         <v>95</v>
       </c>
-      <c r="H6" s="72" t="s">
+      <c r="H6" s="71" t="s">
         <v>114</v>
       </c>
-      <c r="I6" s="73" t="s">
+      <c r="I6" s="72" t="s">
         <v>115</v>
       </c>
       <c r="J6" s="20"/>
@@ -2074,9 +2077,9 @@
       <c r="AB6"/>
       <c r="AC6"/>
     </row>
-    <row r="7" spans="1:29" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="96"/>
-      <c r="B7" s="68" t="s">
+    <row r="7" spans="1:29" ht="51.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="112"/>
+      <c r="B7" s="67" t="s">
         <v>51</v>
       </c>
       <c r="C7" s="9" t="s">
@@ -2091,41 +2094,41 @@
       <c r="F7" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="69" t="s">
+      <c r="G7" s="68" t="s">
         <v>95</v>
       </c>
-      <c r="H7" s="107" t="s">
+      <c r="H7" s="77" t="s">
         <v>114</v>
       </c>
-      <c r="I7" s="120" t="s">
-        <v>139</v>
+      <c r="I7" s="89" t="s">
+        <v>138</v>
       </c>
       <c r="J7" s="20"/>
     </row>
-    <row r="8" spans="1:29" s="7" customFormat="1" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="97"/>
-      <c r="B8" s="51" t="s">
+    <row r="8" spans="1:29" s="7" customFormat="1" ht="48.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="113"/>
+      <c r="B8" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="51" t="s">
+      <c r="C8" s="50" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="70" t="s">
+      <c r="D8" s="69" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="52" t="s">
+      <c r="E8" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="52" t="s">
+      <c r="F8" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="59" t="s">
+      <c r="G8" s="58" t="s">
         <v>95</v>
       </c>
-      <c r="H8" s="54" t="s">
+      <c r="H8" s="53" t="s">
         <v>78</v>
       </c>
-      <c r="I8" s="55"/>
+      <c r="I8" s="54"/>
       <c r="J8" s="20"/>
       <c r="K8"/>
       <c r="L8"/>
@@ -2147,8 +2150,8 @@
       <c r="AB8"/>
       <c r="AC8"/>
     </row>
-    <row r="9" spans="1:29" ht="40.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="64" t="s">
+    <row r="9" spans="1:29" ht="40.5" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="63" t="s">
         <v>21</v>
       </c>
       <c r="B9" s="31" t="s">
@@ -2166,53 +2169,53 @@
       <c r="F9" s="34" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="43" t="s">
+      <c r="G9" s="42" t="s">
         <v>95</v>
       </c>
-      <c r="H9" s="105" t="s">
+      <c r="H9" s="75" t="s">
         <v>114</v>
       </c>
-      <c r="I9" s="106" t="s">
-        <v>138</v>
+      <c r="I9" s="76" t="s">
+        <v>137</v>
       </c>
       <c r="J9" s="20"/>
     </row>
     <row r="10" spans="1:29" ht="42" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="80" t="s">
+      <c r="A10" s="95" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="44" t="s">
+      <c r="B10" s="43" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="44" t="s">
+      <c r="C10" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="66" t="s">
+      <c r="D10" s="65" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="45" t="s">
+      <c r="E10" s="44" t="s">
         <v>60</v>
       </c>
-      <c r="F10" s="45" t="s">
+      <c r="F10" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="G10" s="56" t="s">
+      <c r="G10" s="55" t="s">
         <v>97</v>
       </c>
-      <c r="H10" s="72" t="s">
+      <c r="H10" s="71" t="s">
         <v>114</v>
       </c>
-      <c r="I10" s="49" t="s">
+      <c r="I10" s="48" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:29" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="121"/>
+      <c r="A11" s="96"/>
       <c r="B11" s="32" t="s">
+        <v>143</v>
+      </c>
+      <c r="C11" s="32" t="s">
         <v>144</v>
-      </c>
-      <c r="C11" s="32" t="s">
-        <v>145</v>
       </c>
       <c r="D11" s="33" t="s">
         <v>19</v>
@@ -2223,71 +2226,73 @@
       <c r="F11" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="G11" s="122" t="s">
+      <c r="G11" s="90" t="s">
         <v>97</v>
       </c>
-      <c r="H11" s="42" t="s">
+      <c r="H11" s="75" t="s">
+        <v>114</v>
+      </c>
+      <c r="I11" s="76" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="12" spans="1:29" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="93"/>
+      <c r="B12" s="50" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="51" t="s">
+        <v>98</v>
+      </c>
+      <c r="F12" s="50" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" s="70" t="s">
+        <v>97</v>
+      </c>
+      <c r="H12" s="53" t="s">
         <v>78</v>
       </c>
-      <c r="I11" s="123"/>
-    </row>
-    <row r="12" spans="1:29" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="78"/>
-      <c r="B12" s="51" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="51" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="51" t="s">
+      <c r="I12" s="54"/>
+    </row>
+    <row r="13" spans="1:29" ht="51.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="94" t="s">
+        <v>113</v>
+      </c>
+      <c r="B13" s="43" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="52" t="s">
-        <v>98</v>
-      </c>
-      <c r="F12" s="51" t="s">
-        <v>59</v>
-      </c>
-      <c r="G12" s="71" t="s">
+      <c r="E13" s="44" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" s="45" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" s="55" t="s">
         <v>97</v>
       </c>
-      <c r="H12" s="54" t="s">
-        <v>78</v>
-      </c>
-      <c r="I12" s="55"/>
-    </row>
-    <row r="13" spans="1:29" ht="51.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="79" t="s">
-        <v>113</v>
-      </c>
-      <c r="B13" s="44" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="44" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="F13" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="G13" s="56" t="s">
-        <v>97</v>
-      </c>
-      <c r="H13" s="72" t="s">
+      <c r="H13" s="71" t="s">
         <v>114</v>
       </c>
-      <c r="I13" s="49" t="s">
-        <v>130</v>
+      <c r="I13" s="48" t="s">
+        <v>147</v>
       </c>
       <c r="J13" s="20"/>
     </row>
-    <row r="14" spans="1:29" ht="51" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="77"/>
+    <row r="14" spans="1:29" ht="51" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="92"/>
       <c r="B14" s="11" t="s">
         <v>30</v>
       </c>
@@ -2303,45 +2308,45 @@
       <c r="F14" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="G14" s="57" t="s">
+      <c r="G14" s="56" t="s">
         <v>97</v>
       </c>
-      <c r="H14" s="72" t="s">
+      <c r="H14" s="71" t="s">
         <v>114</v>
       </c>
       <c r="I14" s="19" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J14" s="20"/>
     </row>
-    <row r="15" spans="1:29" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="78"/>
-      <c r="B15" s="51" t="s">
+    <row r="15" spans="1:29" ht="51" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="93"/>
+      <c r="B15" s="50" t="s">
         <v>92</v>
       </c>
-      <c r="C15" s="51" t="s">
+      <c r="C15" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="D15" s="51" t="s">
+      <c r="D15" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="52" t="s">
+      <c r="E15" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="F15" s="58" t="s">
+      <c r="F15" s="57" t="s">
         <v>59</v>
       </c>
-      <c r="G15" s="62" t="s">
+      <c r="G15" s="61" t="s">
         <v>96</v>
       </c>
-      <c r="H15" s="54" t="s">
+      <c r="H15" s="53" t="s">
         <v>78</v>
       </c>
-      <c r="I15" s="55"/>
+      <c r="I15" s="54"/>
       <c r="J15" s="20"/>
     </row>
     <row r="16" spans="1:29" ht="47.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="98" t="s">
+      <c r="A16" s="114" t="s">
         <v>34</v>
       </c>
       <c r="B16" s="13" t="s">
@@ -2353,13 +2358,13 @@
       <c r="D16" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="74" t="s">
+      <c r="E16" s="73" t="s">
         <v>60</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>59</v>
-      </c>
-      <c r="G16" s="56" t="s">
+        <v>145</v>
+      </c>
+      <c r="G16" s="55" t="s">
         <v>97</v>
       </c>
       <c r="H16" s="40" t="s">
@@ -2369,7 +2374,7 @@
       <c r="J16" s="20"/>
     </row>
     <row r="17" spans="1:29" ht="48.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="98"/>
+      <c r="A17" s="114"/>
       <c r="B17" s="13" t="s">
         <v>38</v>
       </c>
@@ -2379,13 +2384,13 @@
       <c r="D17" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="74" t="s">
+      <c r="E17" s="73" t="s">
         <v>60</v>
       </c>
       <c r="F17" s="36" t="s">
-        <v>59</v>
-      </c>
-      <c r="G17" s="56" t="s">
+        <v>145</v>
+      </c>
+      <c r="G17" s="55" t="s">
         <v>97</v>
       </c>
       <c r="H17" s="40" t="s">
@@ -2395,7 +2400,7 @@
       <c r="J17" s="20"/>
     </row>
     <row r="18" spans="1:29" s="7" customFormat="1" ht="51.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="99"/>
+      <c r="A18" s="115"/>
       <c r="B18" s="14" t="s">
         <v>39</v>
       </c>
@@ -2405,13 +2410,13 @@
       <c r="D18" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="75" t="s">
+      <c r="E18" s="74" t="s">
         <v>60</v>
       </c>
-      <c r="F18" s="75" t="s">
-        <v>59</v>
-      </c>
-      <c r="G18" s="56" t="s">
+      <c r="F18" s="74" t="s">
+        <v>145</v>
+      </c>
+      <c r="G18" s="55" t="s">
         <v>97</v>
       </c>
       <c r="H18" s="41" t="s">
@@ -2439,36 +2444,36 @@
       <c r="AB18"/>
       <c r="AC18"/>
     </row>
-    <row r="19" spans="1:29" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="100" t="s">
+    <row r="19" spans="1:29" ht="33" hidden="1" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="116" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="44" t="s">
+      <c r="B19" s="43" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="44" t="s">
+      <c r="C19" s="43" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="44" t="s">
+      <c r="D19" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="45" t="s">
+      <c r="E19" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="F19" s="45" t="s">
+      <c r="F19" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="G19" s="60" t="s">
+      <c r="G19" s="59" t="s">
         <v>96</v>
       </c>
-      <c r="H19" s="72" t="s">
+      <c r="H19" s="71" t="s">
         <v>114</v>
       </c>
-      <c r="I19" s="49"/>
+      <c r="I19" s="48"/>
       <c r="J19" s="20"/>
     </row>
-    <row r="20" spans="1:29" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="77"/>
+    <row r="20" spans="1:29" ht="33" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="92"/>
       <c r="B20" s="11" t="s">
         <v>45</v>
       </c>
@@ -2484,17 +2489,17 @@
       <c r="F20" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G20" s="61" t="s">
+      <c r="G20" s="60" t="s">
         <v>96</v>
       </c>
-      <c r="H20" s="107" t="s">
+      <c r="H20" s="77" t="s">
         <v>114</v>
       </c>
       <c r="I20" s="28"/>
       <c r="J20" s="20"/>
     </row>
-    <row r="21" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="77"/>
+    <row r="21" spans="1:29" ht="48.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="92"/>
       <c r="B21" s="11" t="s">
         <v>41</v>
       </c>
@@ -2510,17 +2515,17 @@
       <c r="F21" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G21" s="61" t="s">
+      <c r="G21" s="60" t="s">
         <v>96</v>
       </c>
-      <c r="H21" s="107" t="s">
+      <c r="H21" s="77" t="s">
         <v>114</v>
       </c>
       <c r="I21" s="19"/>
       <c r="J21" s="20"/>
     </row>
-    <row r="22" spans="1:29" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="77"/>
+    <row r="22" spans="1:29" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="92"/>
       <c r="B22" s="11" t="s">
         <v>42</v>
       </c>
@@ -2536,17 +2541,17 @@
       <c r="F22" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G22" s="61" t="s">
+      <c r="G22" s="60" t="s">
         <v>96</v>
       </c>
-      <c r="H22" s="107" t="s">
+      <c r="H22" s="77" t="s">
         <v>114</v>
       </c>
       <c r="I22" s="19"/>
       <c r="J22" s="20"/>
     </row>
-    <row r="23" spans="1:29" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="77"/>
+    <row r="23" spans="1:29" ht="47.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="92"/>
       <c r="B23" s="11" t="s">
         <v>36</v>
       </c>
@@ -2562,17 +2567,17 @@
       <c r="F23" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G23" s="61" t="s">
+      <c r="G23" s="60" t="s">
         <v>96</v>
       </c>
-      <c r="H23" s="50" t="s">
+      <c r="H23" s="49" t="s">
         <v>78</v>
       </c>
       <c r="I23" s="19"/>
       <c r="J23" s="20"/>
     </row>
-    <row r="24" spans="1:29" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="77"/>
+    <row r="24" spans="1:29" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="92"/>
       <c r="B24" s="11" t="s">
         <v>43</v>
       </c>
@@ -2588,39 +2593,39 @@
       <c r="F24" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G24" s="61" t="s">
+      <c r="G24" s="60" t="s">
         <v>96</v>
       </c>
-      <c r="H24" s="107" t="s">
+      <c r="H24" s="77" t="s">
         <v>114</v>
       </c>
       <c r="I24" s="27"/>
       <c r="J24" s="20"/>
     </row>
-    <row r="25" spans="1:29" s="7" customFormat="1" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="78"/>
-      <c r="B25" s="51" t="s">
+    <row r="25" spans="1:29" s="7" customFormat="1" ht="68.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="93"/>
+      <c r="B25" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="C25" s="51" t="s">
+      <c r="C25" s="50" t="s">
         <v>53</v>
       </c>
-      <c r="D25" s="51" t="s">
+      <c r="D25" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="E25" s="52" t="s">
+      <c r="E25" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="F25" s="52" t="s">
+      <c r="F25" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="G25" s="62" t="s">
+      <c r="G25" s="61" t="s">
         <v>96</v>
       </c>
-      <c r="H25" s="108" t="s">
+      <c r="H25" s="78" t="s">
         <v>114</v>
       </c>
-      <c r="I25" s="55"/>
+      <c r="I25" s="54"/>
       <c r="J25" s="20"/>
       <c r="K25"/>
       <c r="L25"/>
@@ -2643,31 +2648,31 @@
       <c r="AC25"/>
     </row>
     <row r="26" spans="1:29" s="15" customFormat="1" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="92" t="s">
+      <c r="A26" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="B26" s="44" t="s">
+      <c r="B26" s="43" t="s">
         <v>56</v>
       </c>
-      <c r="C26" s="44" t="s">
+      <c r="C26" s="43" t="s">
         <v>61</v>
       </c>
-      <c r="D26" s="44" t="s">
+      <c r="D26" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="E26" s="45" t="s">
+      <c r="E26" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="F26" s="45" t="s">
+      <c r="F26" s="44" t="s">
         <v>59</v>
       </c>
-      <c r="G26" s="56" t="s">
+      <c r="G26" s="55" t="s">
         <v>97</v>
       </c>
-      <c r="H26" s="48" t="s">
+      <c r="H26" s="47" t="s">
         <v>78</v>
       </c>
-      <c r="I26" s="49"/>
+      <c r="I26" s="48"/>
       <c r="J26"/>
       <c r="K26"/>
       <c r="L26"/>
@@ -2690,7 +2695,7 @@
       <c r="AC26"/>
     </row>
     <row r="27" spans="1:29" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="93"/>
+      <c r="A27" s="109"/>
       <c r="B27" s="11" t="s">
         <v>111</v>
       </c>
@@ -2706,39 +2711,39 @@
       <c r="F27" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="G27" s="57" t="s">
+      <c r="G27" s="56" t="s">
         <v>97</v>
       </c>
-      <c r="H27" s="50" t="s">
-        <v>78</v>
+      <c r="H27" s="77" t="s">
+        <v>114</v>
       </c>
       <c r="I27" s="19"/>
     </row>
-    <row r="28" spans="1:29" s="17" customFormat="1" ht="55.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="94"/>
-      <c r="B28" s="51" t="s">
+    <row r="28" spans="1:29" s="17" customFormat="1" ht="55.5" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="110"/>
+      <c r="B28" s="50" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="51" t="s">
+      <c r="C28" s="50" t="s">
         <v>62</v>
       </c>
-      <c r="D28" s="51" t="s">
+      <c r="D28" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="E28" s="52" t="s">
+      <c r="E28" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="F28" s="58" t="s">
+      <c r="F28" s="57" t="s">
         <v>20</v>
       </c>
-      <c r="G28" s="59" t="s">
+      <c r="G28" s="58" t="s">
         <v>95</v>
       </c>
-      <c r="H28" s="108" t="s">
+      <c r="H28" s="78" t="s">
         <v>114</v>
       </c>
-      <c r="I28" s="55" t="s">
-        <v>132</v>
+      <c r="I28" s="54" t="s">
+        <v>131</v>
       </c>
       <c r="J28"/>
       <c r="K28"/>
@@ -2761,37 +2766,37 @@
       <c r="AB28"/>
       <c r="AC28"/>
     </row>
-    <row r="29" spans="1:29" ht="28.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="76" t="s">
+    <row r="29" spans="1:29" ht="28.5" hidden="1" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="91" t="s">
         <v>35</v>
       </c>
-      <c r="B29" s="44" t="s">
+      <c r="B29" s="43" t="s">
         <v>99</v>
       </c>
-      <c r="C29" s="44" t="s">
+      <c r="C29" s="43" t="s">
         <v>104</v>
       </c>
-      <c r="D29" s="44" t="s">
+      <c r="D29" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="E29" s="45" t="s">
+      <c r="E29" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="F29" s="46" t="s">
+      <c r="F29" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="G29" s="47" t="s">
+      <c r="G29" s="46" t="s">
         <v>94</v>
       </c>
-      <c r="H29" s="72" t="s">
+      <c r="H29" s="71" t="s">
         <v>114</v>
       </c>
-      <c r="I29" s="49" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="30" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="77"/>
+      <c r="I29" s="48" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="30" spans="1:29" ht="25.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="92"/>
       <c r="B30" s="11" t="s">
         <v>100</v>
       </c>
@@ -2810,13 +2815,13 @@
       <c r="G30" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="H30" s="50" t="s">
+      <c r="H30" s="49" t="s">
         <v>78</v>
       </c>
       <c r="I30" s="19"/>
     </row>
-    <row r="31" spans="1:29" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="77"/>
+    <row r="31" spans="1:29" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="92"/>
       <c r="B31" s="11" t="s">
         <v>101</v>
       </c>
@@ -2835,13 +2840,13 @@
       <c r="G31" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="H31" s="50" t="s">
+      <c r="H31" s="49" t="s">
         <v>78</v>
       </c>
       <c r="I31" s="19"/>
     </row>
-    <row r="32" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="77"/>
+    <row r="32" spans="1:29" ht="25.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="92"/>
       <c r="B32" s="11" t="s">
         <v>105</v>
       </c>
@@ -2860,13 +2865,13 @@
       <c r="G32" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="H32" s="50" t="s">
+      <c r="H32" s="49" t="s">
         <v>78</v>
       </c>
       <c r="I32" s="19"/>
     </row>
-    <row r="33" spans="1:29" s="16" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="77"/>
+    <row r="33" spans="1:29" s="16" customFormat="1" ht="37.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="92"/>
       <c r="B33" s="11" t="s">
         <v>55</v>
       </c>
@@ -2885,7 +2890,7 @@
       <c r="G33" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="H33" s="50" t="s">
+      <c r="H33" s="49" t="s">
         <v>78</v>
       </c>
       <c r="I33" s="19"/>
@@ -2910,13 +2915,13 @@
       <c r="AB33"/>
       <c r="AC33"/>
     </row>
-    <row r="34" spans="1:29" s="16" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="77"/>
+    <row r="34" spans="1:29" s="16" customFormat="1" ht="37.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="92"/>
       <c r="B34" s="11" t="s">
         <v>26</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>19</v>
@@ -2930,7 +2935,7 @@
       <c r="G34" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="H34" s="50" t="s">
+      <c r="H34" s="49" t="s">
         <v>78</v>
       </c>
       <c r="I34" s="19"/>
@@ -2955,13 +2960,13 @@
       <c r="AB34"/>
       <c r="AC34"/>
     </row>
-    <row r="35" spans="1:29" s="16" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="77"/>
+    <row r="35" spans="1:29" s="16" customFormat="1" ht="37.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="92"/>
       <c r="B35" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="C35" s="11" t="s">
         <v>140</v>
-      </c>
-      <c r="C35" s="11" t="s">
-        <v>141</v>
       </c>
       <c r="D35" s="11" t="s">
         <v>19</v>
@@ -2975,11 +2980,11 @@
       <c r="G35" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="H35" s="107" t="s">
+      <c r="H35" s="77" t="s">
         <v>114</v>
       </c>
       <c r="I35" s="19" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J35"/>
       <c r="K35"/>
@@ -3002,8 +3007,8 @@
       <c r="AB35"/>
       <c r="AC35"/>
     </row>
-    <row r="36" spans="1:29" s="16" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="77"/>
+    <row r="36" spans="1:29" s="16" customFormat="1" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="92"/>
       <c r="B36" s="11" t="s">
         <v>107</v>
       </c>
@@ -3022,7 +3027,7 @@
       <c r="G36" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="H36" s="50" t="s">
+      <c r="H36" s="49" t="s">
         <v>78</v>
       </c>
       <c r="I36" s="19"/>
@@ -3047,30 +3052,30 @@
       <c r="AB36"/>
       <c r="AC36"/>
     </row>
-    <row r="37" spans="1:29" s="16" customFormat="1" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="78"/>
-      <c r="B37" s="51" t="s">
+    <row r="37" spans="1:29" s="16" customFormat="1" ht="33.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="93"/>
+      <c r="B37" s="50" t="s">
         <v>109</v>
       </c>
-      <c r="C37" s="51" t="s">
+      <c r="C37" s="50" t="s">
         <v>110</v>
       </c>
-      <c r="D37" s="51" t="s">
+      <c r="D37" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="E37" s="52" t="s">
+      <c r="E37" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="F37" s="52" t="s">
+      <c r="F37" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="G37" s="53" t="s">
+      <c r="G37" s="52" t="s">
         <v>94</v>
       </c>
-      <c r="H37" s="54" t="s">
+      <c r="H37" s="53" t="s">
         <v>78</v>
       </c>
-      <c r="I37" s="55"/>
+      <c r="I37" s="54"/>
       <c r="J37"/>
       <c r="K37"/>
       <c r="L37"/>
@@ -3092,9 +3097,14 @@
       <c r="AB37"/>
       <c r="AC37"/>
     </row>
-    <row r="38" spans="1:29" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="H5:H37" xr:uid="{4AB4A1F4-D2AB-4474-B05F-C8B13F4E557C}"/>
+  <autoFilter ref="G5:G37" xr:uid="{4AB4A1F4-D2AB-4474-B05F-C8B13F4E557C}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Nathen Reed"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="11">
     <mergeCell ref="A29:A37"/>
     <mergeCell ref="A13:A15"/>
@@ -3132,28 +3142,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="117" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="102"/>
-      <c r="C1" s="102"/>
-      <c r="D1" s="102"/>
-      <c r="E1" s="102"/>
-      <c r="F1" s="102"/>
-      <c r="G1" s="111"/>
+      <c r="B1" s="118"/>
+      <c r="C1" s="118"/>
+      <c r="D1" s="118"/>
+      <c r="E1" s="118"/>
+      <c r="F1" s="118"/>
+      <c r="G1" s="81"/>
     </row>
     <row r="2" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="39" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="103" t="s">
+      <c r="B2" s="119" t="s">
         <v>86</v>
       </c>
-      <c r="C2" s="104"/>
-      <c r="D2" s="104"/>
-      <c r="E2" s="104"/>
-      <c r="F2" s="104"/>
-      <c r="G2" s="112"/>
+      <c r="C2" s="120"/>
+      <c r="D2" s="120"/>
+      <c r="E2" s="120"/>
+      <c r="F2" s="120"/>
+      <c r="G2" s="82"/>
     </row>
     <row r="3" spans="1:8" s="26" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
@@ -3171,223 +3181,223 @@
       <c r="E3" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="109" t="s">
+      <c r="F3" s="79" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="113" t="s">
+      <c r="G3" s="83" t="s">
         <v>88</v>
       </c>
-      <c r="H3" s="110"/>
+      <c r="H3" s="80"/>
     </row>
     <row r="4" spans="1:8" ht="225.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="114" t="s">
+      <c r="A4" s="84" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="114" t="s">
+      <c r="B4" s="84" t="s">
         <v>87</v>
       </c>
-      <c r="C4" s="115" t="s">
+      <c r="C4" s="85" t="s">
         <v>124</v>
       </c>
-      <c r="D4" s="114" t="s">
+      <c r="D4" s="84" t="s">
         <v>125</v>
       </c>
-      <c r="E4" s="114" t="s">
+      <c r="E4" s="84" t="s">
         <v>126</v>
       </c>
-      <c r="F4" s="114" t="s">
+      <c r="F4" s="84" t="s">
         <v>127</v>
       </c>
-      <c r="G4" s="114" t="s">
+      <c r="G4" s="84" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="143.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="114" t="s">
+      <c r="A5" s="84" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="114" t="s">
+      <c r="B5" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="115" t="s">
+      <c r="C5" s="85" t="s">
         <v>85</v>
       </c>
-      <c r="D5" s="114" t="s">
+      <c r="D5" s="84" t="s">
+        <v>132</v>
+      </c>
+      <c r="E5" s="84" t="s">
         <v>133</v>
       </c>
-      <c r="E5" s="114" t="s">
+      <c r="F5" s="84" t="s">
         <v>134</v>
       </c>
-      <c r="F5" s="114" t="s">
+      <c r="G5" s="84" t="s">
         <v>135</v>
       </c>
-      <c r="G5" s="114" t="s">
-        <v>136</v>
-      </c>
     </row>
     <row r="6" spans="1:8" ht="191.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="114" t="s">
+      <c r="A6" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="114" t="s">
+      <c r="B6" s="84" t="s">
         <v>66</v>
       </c>
-      <c r="C6" s="115" t="s">
+      <c r="C6" s="85" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="114"/>
-      <c r="E6" s="114"/>
-      <c r="F6" s="114"/>
-      <c r="G6" s="114"/>
+      <c r="D6" s="84"/>
+      <c r="E6" s="84"/>
+      <c r="F6" s="84"/>
+      <c r="G6" s="84"/>
     </row>
     <row r="7" spans="1:8" ht="115.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="114" t="s">
+      <c r="A7" s="84" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="114" t="s">
+      <c r="B7" s="84" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="115" t="s">
+      <c r="C7" s="85" t="s">
         <v>85</v>
       </c>
-      <c r="D7" s="114"/>
-      <c r="E7" s="114"/>
-      <c r="F7" s="114"/>
-      <c r="G7" s="114"/>
+      <c r="D7" s="84"/>
+      <c r="E7" s="84"/>
+      <c r="F7" s="84"/>
+      <c r="G7" s="84"/>
     </row>
     <row r="8" spans="1:8" s="29" customFormat="1" ht="227.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="116" t="s">
+      <c r="A8" s="86" t="s">
         <v>72</v>
       </c>
-      <c r="B8" s="117" t="s">
+      <c r="B8" s="121" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="115" t="s">
+      <c r="C8" s="85" t="s">
         <v>85</v>
       </c>
-      <c r="D8" s="114"/>
-      <c r="E8" s="118"/>
-      <c r="F8" s="114"/>
-      <c r="G8" s="114"/>
+      <c r="D8" s="84"/>
+      <c r="E8" s="87"/>
+      <c r="F8" s="84"/>
+      <c r="G8" s="84"/>
     </row>
     <row r="9" spans="1:8" ht="238.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="114" t="s">
+      <c r="A9" s="84" t="s">
         <v>68</v>
       </c>
-      <c r="B9" s="117"/>
-      <c r="C9" s="115" t="s">
+      <c r="B9" s="121"/>
+      <c r="C9" s="85" t="s">
         <v>85</v>
       </c>
-      <c r="D9" s="114"/>
-      <c r="E9" s="118"/>
-      <c r="F9" s="114"/>
-      <c r="G9" s="114"/>
+      <c r="D9" s="84"/>
+      <c r="E9" s="87"/>
+      <c r="F9" s="84"/>
+      <c r="G9" s="84"/>
     </row>
     <row r="10" spans="1:8" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="119" t="s">
+      <c r="A10" s="88" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="117"/>
-      <c r="C10" s="119" t="s">
+      <c r="B10" s="121"/>
+      <c r="C10" s="88" t="s">
         <v>85</v>
       </c>
-      <c r="D10" s="119"/>
-      <c r="E10" s="118"/>
-      <c r="F10" s="114"/>
-      <c r="G10" s="114"/>
+      <c r="D10" s="88"/>
+      <c r="E10" s="87"/>
+      <c r="F10" s="84"/>
+      <c r="G10" s="84"/>
     </row>
     <row r="11" spans="1:8" ht="145.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="114" t="s">
+      <c r="A11" s="84" t="s">
         <v>70</v>
       </c>
-      <c r="B11" s="117"/>
-      <c r="C11" s="115" t="s">
+      <c r="B11" s="121"/>
+      <c r="C11" s="85" t="s">
         <v>85</v>
       </c>
-      <c r="D11" s="114"/>
-      <c r="E11" s="118"/>
-      <c r="F11" s="114"/>
-      <c r="G11" s="114"/>
+      <c r="D11" s="84"/>
+      <c r="E11" s="87"/>
+      <c r="F11" s="84"/>
+      <c r="G11" s="84"/>
     </row>
     <row r="12" spans="1:8" s="30" customFormat="1" ht="102" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="114" t="s">
+      <c r="A12" s="84" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="117"/>
-      <c r="C12" s="115" t="s">
+      <c r="B12" s="121"/>
+      <c r="C12" s="85" t="s">
         <v>85</v>
       </c>
-      <c r="D12" s="114"/>
-      <c r="E12" s="118"/>
-      <c r="F12" s="114"/>
-      <c r="G12" s="114"/>
+      <c r="D12" s="84"/>
+      <c r="E12" s="87"/>
+      <c r="F12" s="84"/>
+      <c r="G12" s="84"/>
     </row>
     <row r="13" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="114" t="s">
+      <c r="A13" s="84" t="s">
         <v>116</v>
       </c>
-      <c r="B13" s="114" t="s">
+      <c r="B13" s="84" t="s">
         <v>119</v>
       </c>
-      <c r="C13" s="115" t="s">
+      <c r="C13" s="85" t="s">
         <v>85</v>
       </c>
-      <c r="D13" s="114"/>
-      <c r="E13" s="114"/>
-      <c r="F13" s="114"/>
-      <c r="G13" s="114"/>
+      <c r="D13" s="84"/>
+      <c r="E13" s="84"/>
+      <c r="F13" s="84"/>
+      <c r="G13" s="84"/>
     </row>
     <row r="14" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="114" t="s">
+      <c r="A14" s="84" t="s">
         <v>117</v>
       </c>
-      <c r="B14" s="114" t="s">
+      <c r="B14" s="84" t="s">
         <v>120</v>
       </c>
-      <c r="C14" s="115" t="s">
+      <c r="C14" s="85" t="s">
         <v>85</v>
       </c>
-      <c r="D14" s="114"/>
-      <c r="E14" s="114"/>
-      <c r="F14" s="114"/>
-      <c r="G14" s="114"/>
+      <c r="D14" s="84"/>
+      <c r="E14" s="84"/>
+      <c r="F14" s="84"/>
+      <c r="G14" s="84"/>
     </row>
     <row r="15" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="114" t="s">
+      <c r="A15" s="84" t="s">
         <v>118</v>
       </c>
-      <c r="B15" s="114" t="s">
+      <c r="B15" s="84" t="s">
         <v>121</v>
       </c>
-      <c r="C15" s="115" t="s">
+      <c r="C15" s="85" t="s">
         <v>85</v>
       </c>
-      <c r="D15" s="114"/>
-      <c r="E15" s="114"/>
-      <c r="F15" s="114"/>
-      <c r="G15" s="114"/>
+      <c r="D15" s="84"/>
+      <c r="E15" s="84"/>
+      <c r="F15" s="84"/>
+      <c r="G15" s="84"/>
     </row>
     <row r="16" spans="1:8" ht="84" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="114" t="s">
+      <c r="A16" s="84" t="s">
         <v>122</v>
       </c>
-      <c r="B16" s="114" t="s">
+      <c r="B16" s="84" t="s">
         <v>123</v>
       </c>
-      <c r="C16" s="114"/>
-      <c r="D16" s="114"/>
-      <c r="E16" s="114"/>
-      <c r="F16" s="114"/>
-      <c r="G16" s="114"/>
+      <c r="C16" s="84"/>
+      <c r="D16" s="84"/>
+      <c r="E16" s="84"/>
+      <c r="F16" s="84"/>
+      <c r="G16" s="84"/>
     </row>
     <row r="17" spans="1:7" ht="99.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="114"/>
-      <c r="B17" s="114"/>
-      <c r="C17" s="114"/>
-      <c r="D17" s="114"/>
-      <c r="E17" s="114"/>
-      <c r="F17" s="114"/>
-      <c r="G17" s="114"/>
+      <c r="A17" s="84"/>
+      <c r="B17" s="84"/>
+      <c r="C17" s="84"/>
+      <c r="D17" s="84"/>
+      <c r="E17" s="84"/>
+      <c r="F17" s="84"/>
+      <c r="G17" s="84"/>
     </row>
     <row r="18" spans="1:7" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="21"/>
@@ -3764,6 +3774,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="ff8a4b2e-b0c8-4039-a689-d1a7f36f4382">
@@ -3773,15 +3792,6 @@
     <Notes xmlns="ff8a4b2e-b0c8-4039-a689-d1a7f36f4382" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3804,6 +3814,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8F3069D-89E7-4007-93BF-1DB2942FF756}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76F271AB-EFB2-4823-A2F0-9F2289E658DB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3814,12 +3832,4 @@
     <ds:schemaRef ds:uri="f716dd8a-49a0-4c40-b209-038e1651b548"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8F3069D-89E7-4007-93BF-1DB2942FF756}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Final Beta, Adjusted enemy classes and collision channel
</commit_message>
<xml_diff>
--- a/Red Team Tracebility and Testing.xlsx
+++ b/Red Team Tracebility and Testing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Program Files\Epic Games\UE_5.7\redteam\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8409E52F-DFBA-4DAB-AB3C-531532A5DFE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4472431A-0CCB-4D31-AD20-F02E702BD0A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{19EF330C-6F54-4365-A47E-10806019DE9B}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Test Plan" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Traceability Matrix'!$G$5:$G$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Traceability Matrix'!$G$5:$G$36</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="150">
   <si>
     <t>Prototype Title:</t>
   </si>
@@ -121,9 +121,6 @@
   </si>
   <si>
     <t>Collectible Items</t>
-  </si>
-  <si>
-    <t>Small valuable items that fit into inventory.</t>
   </si>
   <si>
     <t>Health kits that are collected by player to regain health when needed.</t>
@@ -425,9 +422,6 @@
     <t>Nathen Reed</t>
   </si>
   <si>
-    <t xml:space="preserve"> Alpha</t>
-  </si>
-  <si>
     <t>Player Design</t>
   </si>
   <si>
@@ -573,6 +567,18 @@
   </si>
   <si>
     <t>Checkpoint Updated With custom FB. -Nathen Reed</t>
+  </si>
+  <si>
+    <t>Created levels 1 and 2 pending final third level. -Nathen Reed</t>
+  </si>
+  <si>
+    <t>Added simple moving platform that ping pongs between two spots. -Nathen Reed</t>
+  </si>
+  <si>
+    <t>Added long/short jump and double jump -Nathen Reed</t>
+  </si>
+  <si>
+    <t>Added but needs som small adjustments to projectile.</t>
   </si>
 </sst>
 </file>
@@ -1267,7 +1273,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1401,7 +1407,6 @@
     <xf numFmtId="0" fontId="6" fillId="12" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1444,9 +1449,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1914,7 +1916,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB4A1F4-D2AB-4474-B05F-C8B13F4E557C}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AC37"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1926,35 +1927,35 @@
     <col min="6" max="6" width="16.85546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="13" style="1" customWidth="1"/>
     <col min="8" max="8" width="17.5703125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="53.85546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="69.5703125" style="1" customWidth="1"/>
     <col min="10" max="12" width="23.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="100" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="101"/>
-      <c r="I1" s="101"/>
+      <c r="A1" s="98" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="99"/>
+      <c r="C1" s="99"/>
+      <c r="D1" s="99"/>
+      <c r="E1" s="99"/>
+      <c r="F1" s="99"/>
+      <c r="G1" s="99"/>
+      <c r="H1" s="99"/>
+      <c r="I1" s="99"/>
     </row>
     <row r="2" spans="1:29" s="3" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="97"/>
-      <c r="C2" s="98"/>
-      <c r="D2" s="98"/>
-      <c r="E2" s="98"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="98"/>
-      <c r="I2" s="99"/>
+      <c r="B2" s="95"/>
+      <c r="C2" s="96"/>
+      <c r="D2" s="96"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="96"/>
+      <c r="G2" s="96"/>
+      <c r="H2" s="96"/>
+      <c r="I2" s="97"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
@@ -1973,88 +1974,88 @@
       <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="102" t="s">
-        <v>84</v>
-      </c>
-      <c r="C3" s="103"/>
-      <c r="D3" s="103"/>
-      <c r="E3" s="103"/>
-      <c r="F3" s="103"/>
-      <c r="G3" s="103"/>
-      <c r="H3" s="103"/>
-      <c r="I3" s="104"/>
+      <c r="B3" s="100" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3" s="101"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="102"/>
     </row>
     <row r="4" spans="1:29" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="38" t="s">
-        <v>83</v>
-      </c>
-      <c r="B4" s="105" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" s="106"/>
-      <c r="D4" s="106"/>
-      <c r="E4" s="106"/>
-      <c r="F4" s="106"/>
-      <c r="G4" s="106"/>
-      <c r="H4" s="106"/>
-      <c r="I4" s="107"/>
+        <v>82</v>
+      </c>
+      <c r="B4" s="103" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" s="104"/>
+      <c r="D4" s="104"/>
+      <c r="E4" s="104"/>
+      <c r="F4" s="104"/>
+      <c r="G4" s="104"/>
+      <c r="H4" s="104"/>
+      <c r="I4" s="105"/>
     </row>
     <row r="5" spans="1:29" s="2" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="62" t="s">
+      <c r="A5" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="62" t="s">
+      <c r="B5" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="62" t="s">
+      <c r="C5" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="62" t="s">
+      <c r="D5" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="62" t="s">
+      <c r="E5" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="62" t="s">
+      <c r="F5" s="61" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="62" t="s">
+      <c r="G5" s="61" t="s">
         <v>15</v>
       </c>
       <c r="H5" s="35" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I5" s="35" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="6" spans="1:29" s="8" customFormat="1" ht="46.5" hidden="1" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="111" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" s="8" customFormat="1" ht="46.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="109" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="64" t="s">
+      <c r="B6" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="65" t="s">
-        <v>81</v>
-      </c>
-      <c r="D6" s="65" t="s">
+      <c r="C6" s="64" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" s="64" t="s">
         <v>19</v>
       </c>
       <c r="E6" s="44" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F6" s="45" t="s">
-        <v>33</v>
-      </c>
-      <c r="G6" s="66" t="s">
-        <v>95</v>
-      </c>
-      <c r="H6" s="71" t="s">
-        <v>114</v>
-      </c>
-      <c r="I6" s="72" t="s">
-        <v>115</v>
+        <v>32</v>
+      </c>
+      <c r="G6" s="65" t="s">
+        <v>94</v>
+      </c>
+      <c r="H6" s="69" t="s">
+        <v>112</v>
+      </c>
+      <c r="I6" s="70" t="s">
+        <v>113</v>
       </c>
       <c r="J6" s="20"/>
       <c r="K6"/>
@@ -2077,58 +2078,60 @@
       <c r="AB6"/>
       <c r="AC6"/>
     </row>
-    <row r="7" spans="1:29" ht="51.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="112"/>
-      <c r="B7" s="67" t="s">
+    <row r="7" spans="1:29" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="110"/>
+      <c r="B7" s="66" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>51</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>52</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>19</v>
       </c>
       <c r="E7" s="36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F7" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="68" t="s">
-        <v>95</v>
-      </c>
-      <c r="H7" s="77" t="s">
-        <v>114</v>
-      </c>
-      <c r="I7" s="89" t="s">
-        <v>138</v>
+      <c r="G7" s="67" t="s">
+        <v>94</v>
+      </c>
+      <c r="H7" s="75" t="s">
+        <v>112</v>
+      </c>
+      <c r="I7" s="87" t="s">
+        <v>136</v>
       </c>
       <c r="J7" s="20"/>
     </row>
-    <row r="8" spans="1:29" s="7" customFormat="1" ht="48.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="113"/>
+    <row r="8" spans="1:29" s="7" customFormat="1" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="111"/>
       <c r="B8" s="50" t="s">
         <v>22</v>
       </c>
       <c r="C8" s="50" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="69" t="s">
+      <c r="D8" s="68" t="s">
         <v>19</v>
       </c>
       <c r="E8" s="51" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F8" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="H8" s="53" t="s">
-        <v>78</v>
-      </c>
-      <c r="I8" s="54"/>
+      <c r="G8" s="57" t="s">
+        <v>94</v>
+      </c>
+      <c r="H8" s="76" t="s">
+        <v>112</v>
+      </c>
+      <c r="I8" s="53" t="s">
+        <v>148</v>
+      </c>
       <c r="J8" s="20"/>
       <c r="K8"/>
       <c r="L8"/>
@@ -2150,356 +2153,357 @@
       <c r="AB8"/>
       <c r="AC8"/>
     </row>
-    <row r="9" spans="1:29" ht="40.5" hidden="1" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="63" t="s">
+    <row r="9" spans="1:29" ht="40.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="62" t="s">
         <v>21</v>
       </c>
       <c r="B9" s="31" t="s">
+        <v>78</v>
+      </c>
+      <c r="C9" s="32" t="s">
         <v>79</v>
-      </c>
-      <c r="C9" s="32" t="s">
-        <v>80</v>
       </c>
       <c r="D9" s="33" t="s">
         <v>19</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F9" s="34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G9" s="42" t="s">
-        <v>95</v>
-      </c>
-      <c r="H9" s="75" t="s">
-        <v>114</v>
-      </c>
-      <c r="I9" s="76" t="s">
-        <v>137</v>
+        <v>94</v>
+      </c>
+      <c r="H9" s="73" t="s">
+        <v>112</v>
+      </c>
+      <c r="I9" s="74" t="s">
+        <v>135</v>
       </c>
       <c r="J9" s="20"/>
     </row>
     <row r="10" spans="1:29" ht="42" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="95" t="s">
+      <c r="A10" s="93" t="s">
         <v>24</v>
       </c>
       <c r="B10" s="43" t="s">
         <v>25</v>
       </c>
       <c r="C10" s="43" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="65" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="64" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="44" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F10" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="G10" s="55" t="s">
-        <v>97</v>
-      </c>
-      <c r="H10" s="71" t="s">
-        <v>114</v>
+      <c r="G10" s="54" t="s">
+        <v>96</v>
+      </c>
+      <c r="H10" s="69" t="s">
+        <v>112</v>
       </c>
       <c r="I10" s="48" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="11" spans="1:29" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="96"/>
+        <v>127</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="94"/>
       <c r="B11" s="32" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C11" s="32" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D11" s="33" t="s">
         <v>19</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F11" s="34" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" s="88" t="s">
+        <v>96</v>
+      </c>
+      <c r="H11" s="73" t="s">
+        <v>112</v>
+      </c>
+      <c r="I11" s="74" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="12" spans="1:29" ht="51.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="92" t="s">
+        <v>111</v>
+      </c>
+      <c r="B12" s="43" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="43" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="44" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="45" t="s">
+        <v>20</v>
+      </c>
+      <c r="G12" s="54" t="s">
+        <v>96</v>
+      </c>
+      <c r="H12" s="69" t="s">
+        <v>112</v>
+      </c>
+      <c r="I12" s="48" t="s">
+        <v>145</v>
+      </c>
+      <c r="J12" s="20"/>
+    </row>
+    <row r="13" spans="1:29" ht="51" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="90"/>
+      <c r="B13" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="G13" s="55" t="s">
+        <v>96</v>
+      </c>
+      <c r="H13" s="69" t="s">
+        <v>112</v>
+      </c>
+      <c r="I13" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="J13" s="20"/>
+    </row>
+    <row r="14" spans="1:29" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="91"/>
+      <c r="B14" s="50" t="s">
+        <v>91</v>
+      </c>
+      <c r="C14" s="50" t="s">
+        <v>92</v>
+      </c>
+      <c r="D14" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="56" t="s">
+        <v>58</v>
+      </c>
+      <c r="G14" s="60" t="s">
+        <v>95</v>
+      </c>
+      <c r="H14" s="76" t="s">
+        <v>112</v>
+      </c>
+      <c r="I14" s="53"/>
+      <c r="J14" s="20"/>
+    </row>
+    <row r="15" spans="1:29" ht="47.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="112" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="71" t="s">
         <v>59</v>
       </c>
-      <c r="G11" s="90" t="s">
-        <v>97</v>
-      </c>
-      <c r="H11" s="75" t="s">
-        <v>114</v>
-      </c>
-      <c r="I11" s="76" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="12" spans="1:29" ht="42.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="93"/>
-      <c r="B12" s="50" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="50" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="50" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="51" t="s">
-        <v>98</v>
-      </c>
-      <c r="F12" s="50" t="s">
-        <v>59</v>
-      </c>
-      <c r="G12" s="70" t="s">
-        <v>97</v>
-      </c>
-      <c r="H12" s="53" t="s">
-        <v>78</v>
-      </c>
-      <c r="I12" s="54"/>
-    </row>
-    <row r="13" spans="1:29" ht="51.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="94" t="s">
-        <v>113</v>
-      </c>
-      <c r="B13" s="43" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="43" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="43" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="44" t="s">
-        <v>33</v>
-      </c>
-      <c r="F13" s="45" t="s">
-        <v>20</v>
-      </c>
-      <c r="G13" s="55" t="s">
-        <v>97</v>
-      </c>
-      <c r="H13" s="71" t="s">
-        <v>114</v>
-      </c>
-      <c r="I13" s="48" t="s">
-        <v>147</v>
-      </c>
-      <c r="J13" s="20"/>
-    </row>
-    <row r="14" spans="1:29" ht="51" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="92"/>
-      <c r="B14" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="36" t="s">
-        <v>33</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="G14" s="56" t="s">
-        <v>97</v>
-      </c>
-      <c r="H14" s="71" t="s">
-        <v>114</v>
-      </c>
-      <c r="I14" s="19" t="s">
-        <v>130</v>
-      </c>
-      <c r="J14" s="20"/>
-    </row>
-    <row r="15" spans="1:29" ht="51" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="93"/>
-      <c r="B15" s="50" t="s">
-        <v>92</v>
-      </c>
-      <c r="C15" s="50" t="s">
-        <v>93</v>
-      </c>
-      <c r="D15" s="50" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="51" t="s">
-        <v>20</v>
-      </c>
-      <c r="F15" s="57" t="s">
-        <v>59</v>
-      </c>
-      <c r="G15" s="61" t="s">
+      <c r="F15" s="36" t="s">
+        <v>143</v>
+      </c>
+      <c r="G15" s="54" t="s">
         <v>96</v>
       </c>
-      <c r="H15" s="53" t="s">
-        <v>78</v>
-      </c>
-      <c r="I15" s="54"/>
+      <c r="H15" s="40" t="s">
+        <v>77</v>
+      </c>
+      <c r="I15" s="19"/>
       <c r="J15" s="20"/>
     </row>
-    <row r="16" spans="1:29" ht="47.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="114" t="s">
-        <v>34</v>
-      </c>
+    <row r="16" spans="1:29" ht="48.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="112"/>
       <c r="B16" s="13" t="s">
         <v>37</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="73" t="s">
-        <v>60</v>
+      <c r="E16" s="71" t="s">
+        <v>59</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="G16" s="55" t="s">
-        <v>97</v>
+        <v>143</v>
+      </c>
+      <c r="G16" s="54" t="s">
+        <v>96</v>
       </c>
       <c r="H16" s="40" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I16" s="19"/>
       <c r="J16" s="20"/>
     </row>
-    <row r="17" spans="1:29" ht="48.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="114"/>
-      <c r="B17" s="13" t="s">
+    <row r="17" spans="1:29" s="7" customFormat="1" ht="51.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="113"/>
+      <c r="B17" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="73" t="s">
-        <v>60</v>
-      </c>
-      <c r="F17" s="36" t="s">
-        <v>145</v>
-      </c>
-      <c r="G17" s="55" t="s">
-        <v>97</v>
-      </c>
-      <c r="H17" s="40" t="s">
-        <v>78</v>
-      </c>
-      <c r="I17" s="19"/>
+      <c r="E17" s="72" t="s">
+        <v>59</v>
+      </c>
+      <c r="F17" s="72" t="s">
+        <v>143</v>
+      </c>
+      <c r="G17" s="54" t="s">
+        <v>96</v>
+      </c>
+      <c r="H17" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="I17" s="18"/>
       <c r="J17" s="20"/>
-    </row>
-    <row r="18" spans="1:29" s="7" customFormat="1" ht="51.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="115"/>
-      <c r="B18" s="14" t="s">
+      <c r="K17"/>
+      <c r="L17"/>
+      <c r="M17"/>
+      <c r="N17"/>
+      <c r="O17"/>
+      <c r="P17"/>
+      <c r="Q17"/>
+      <c r="R17"/>
+      <c r="S17"/>
+      <c r="T17"/>
+      <c r="U17"/>
+      <c r="V17"/>
+      <c r="W17"/>
+      <c r="X17"/>
+      <c r="Y17"/>
+      <c r="Z17"/>
+      <c r="AA17"/>
+      <c r="AB17"/>
+      <c r="AC17"/>
+    </row>
+    <row r="18" spans="1:29" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="114" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="43" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="D18" s="12" t="s">
+      <c r="C18" s="43" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="74" t="s">
-        <v>60</v>
-      </c>
-      <c r="F18" s="74" t="s">
-        <v>145</v>
-      </c>
-      <c r="G18" s="55" t="s">
-        <v>97</v>
-      </c>
-      <c r="H18" s="41" t="s">
-        <v>78</v>
-      </c>
-      <c r="I18" s="18"/>
+      <c r="E18" s="44" t="s">
+        <v>32</v>
+      </c>
+      <c r="F18" s="44" t="s">
+        <v>20</v>
+      </c>
+      <c r="G18" s="58" t="s">
+        <v>95</v>
+      </c>
+      <c r="H18" s="69" t="s">
+        <v>112</v>
+      </c>
+      <c r="I18" s="48"/>
       <c r="J18" s="20"/>
-      <c r="K18"/>
-      <c r="L18"/>
-      <c r="M18"/>
-      <c r="N18"/>
-      <c r="O18"/>
-      <c r="P18"/>
-      <c r="Q18"/>
-      <c r="R18"/>
-      <c r="S18"/>
-      <c r="T18"/>
-      <c r="U18"/>
-      <c r="V18"/>
-      <c r="W18"/>
-      <c r="X18"/>
-      <c r="Y18"/>
-      <c r="Z18"/>
-      <c r="AA18"/>
-      <c r="AB18"/>
-      <c r="AC18"/>
-    </row>
-    <row r="19" spans="1:29" ht="33" hidden="1" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="116" t="s">
-        <v>16</v>
-      </c>
-      <c r="B19" s="43" t="s">
+    </row>
+    <row r="19" spans="1:29" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="90"/>
+      <c r="B19" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="G19" s="59" t="s">
+        <v>95</v>
+      </c>
+      <c r="H19" s="75" t="s">
+        <v>112</v>
+      </c>
+      <c r="I19" s="28"/>
+      <c r="J19" s="20"/>
+    </row>
+    <row r="20" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="90"/>
+      <c r="B20" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="43" t="s">
+      <c r="C20" s="11" t="s">
         <v>46</v>
-      </c>
-      <c r="D19" s="43" t="s">
-        <v>19</v>
-      </c>
-      <c r="E19" s="44" t="s">
-        <v>33</v>
-      </c>
-      <c r="F19" s="44" t="s">
-        <v>20</v>
-      </c>
-      <c r="G19" s="59" t="s">
-        <v>96</v>
-      </c>
-      <c r="H19" s="71" t="s">
-        <v>114</v>
-      </c>
-      <c r="I19" s="48"/>
-      <c r="J19" s="20"/>
-    </row>
-    <row r="20" spans="1:29" ht="33" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="92"/>
-      <c r="B20" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>77</v>
       </c>
       <c r="D20" s="11" t="s">
         <v>19</v>
       </c>
       <c r="E20" s="36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F20" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G20" s="60" t="s">
-        <v>96</v>
-      </c>
-      <c r="H20" s="77" t="s">
-        <v>114</v>
-      </c>
-      <c r="I20" s="28"/>
+      <c r="G20" s="59" t="s">
+        <v>95</v>
+      </c>
+      <c r="H20" s="75" t="s">
+        <v>112</v>
+      </c>
+      <c r="I20" s="19"/>
       <c r="J20" s="20"/>
     </row>
-    <row r="21" spans="1:29" ht="48.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="92"/>
+    <row r="21" spans="1:29" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="90"/>
       <c r="B21" s="11" t="s">
         <v>41</v>
       </c>
@@ -2510,123 +2514,148 @@
         <v>19</v>
       </c>
       <c r="E21" s="36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F21" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G21" s="60" t="s">
-        <v>96</v>
-      </c>
-      <c r="H21" s="77" t="s">
-        <v>114</v>
+      <c r="G21" s="59" t="s">
+        <v>95</v>
+      </c>
+      <c r="H21" s="75" t="s">
+        <v>112</v>
       </c>
       <c r="I21" s="19"/>
       <c r="J21" s="20"/>
     </row>
-    <row r="22" spans="1:29" ht="43.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="92"/>
+    <row r="22" spans="1:29" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="90"/>
       <c r="B22" s="11" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D22" s="11" t="s">
         <v>19</v>
       </c>
       <c r="E22" s="36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F22" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G22" s="60" t="s">
-        <v>96</v>
-      </c>
-      <c r="H22" s="77" t="s">
-        <v>114</v>
-      </c>
-      <c r="I22" s="19"/>
+      <c r="G22" s="59" t="s">
+        <v>95</v>
+      </c>
+      <c r="H22" s="75" t="s">
+        <v>112</v>
+      </c>
+      <c r="I22" s="19" t="s">
+        <v>149</v>
+      </c>
       <c r="J22" s="20"/>
     </row>
-    <row r="23" spans="1:29" ht="47.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="92"/>
+    <row r="23" spans="1:29" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="90"/>
       <c r="B23" s="11" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D23" s="11" t="s">
         <v>19</v>
       </c>
       <c r="E23" s="36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F23" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G23" s="60" t="s">
+      <c r="G23" s="59" t="s">
+        <v>95</v>
+      </c>
+      <c r="H23" s="75" t="s">
+        <v>112</v>
+      </c>
+      <c r="I23" s="27"/>
+      <c r="J23" s="20"/>
+    </row>
+    <row r="24" spans="1:29" s="7" customFormat="1" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="91"/>
+      <c r="B24" s="50" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" s="50" t="s">
+        <v>52</v>
+      </c>
+      <c r="D24" s="50" t="s">
+        <v>19</v>
+      </c>
+      <c r="E24" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="F24" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="G24" s="60" t="s">
+        <v>95</v>
+      </c>
+      <c r="H24" s="76" t="s">
+        <v>112</v>
+      </c>
+      <c r="I24" s="53"/>
+      <c r="J24" s="20"/>
+      <c r="K24"/>
+      <c r="L24"/>
+      <c r="M24"/>
+      <c r="N24"/>
+      <c r="O24"/>
+      <c r="P24"/>
+      <c r="Q24"/>
+      <c r="R24"/>
+      <c r="S24"/>
+      <c r="T24"/>
+      <c r="U24"/>
+      <c r="V24"/>
+      <c r="W24"/>
+      <c r="X24"/>
+      <c r="Y24"/>
+      <c r="Z24"/>
+      <c r="AA24"/>
+      <c r="AB24"/>
+      <c r="AC24"/>
+    </row>
+    <row r="25" spans="1:29" s="15" customFormat="1" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="106" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="43" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" s="43" t="s">
+        <v>60</v>
+      </c>
+      <c r="D25" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="E25" s="44" t="s">
+        <v>32</v>
+      </c>
+      <c r="F25" s="44" t="s">
+        <v>58</v>
+      </c>
+      <c r="G25" s="54" t="s">
         <v>96</v>
       </c>
-      <c r="H23" s="49" t="s">
-        <v>78</v>
-      </c>
-      <c r="I23" s="19"/>
-      <c r="J23" s="20"/>
-    </row>
-    <row r="24" spans="1:29" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="92"/>
-      <c r="B24" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E24" s="36" t="s">
-        <v>33</v>
-      </c>
-      <c r="F24" s="36" t="s">
-        <v>20</v>
-      </c>
-      <c r="G24" s="60" t="s">
-        <v>96</v>
-      </c>
-      <c r="H24" s="77" t="s">
-        <v>114</v>
-      </c>
-      <c r="I24" s="27"/>
-      <c r="J24" s="20"/>
-    </row>
-    <row r="25" spans="1:29" s="7" customFormat="1" ht="68.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="93"/>
-      <c r="B25" s="50" t="s">
-        <v>44</v>
-      </c>
-      <c r="C25" s="50" t="s">
-        <v>53</v>
-      </c>
-      <c r="D25" s="50" t="s">
-        <v>19</v>
-      </c>
-      <c r="E25" s="51" t="s">
-        <v>33</v>
-      </c>
-      <c r="F25" s="51" t="s">
-        <v>20</v>
-      </c>
-      <c r="G25" s="61" t="s">
-        <v>96</v>
-      </c>
-      <c r="H25" s="78" t="s">
-        <v>114</v>
-      </c>
-      <c r="I25" s="54"/>
-      <c r="J25" s="20"/>
+      <c r="H25" s="47" t="s">
+        <v>77</v>
+      </c>
+      <c r="I25" s="48" t="s">
+        <v>146</v>
+      </c>
+      <c r="J25"/>
       <c r="K25"/>
       <c r="L25"/>
       <c r="M25"/>
@@ -2647,251 +2676,251 @@
       <c r="AB25"/>
       <c r="AC25"/>
     </row>
-    <row r="26" spans="1:29" s="15" customFormat="1" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="108" t="s">
-        <v>54</v>
-      </c>
-      <c r="B26" s="43" t="s">
+    <row r="26" spans="1:29" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="107"/>
+      <c r="B26" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="G26" s="55" t="s">
+        <v>96</v>
+      </c>
+      <c r="H26" s="75" t="s">
+        <v>112</v>
+      </c>
+      <c r="I26" s="19" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="27" spans="1:29" s="17" customFormat="1" ht="55.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="108"/>
+      <c r="B27" s="50" t="s">
         <v>56</v>
       </c>
-      <c r="C26" s="43" t="s">
+      <c r="C27" s="50" t="s">
         <v>61</v>
       </c>
-      <c r="D26" s="43" t="s">
+      <c r="D27" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="E26" s="44" t="s">
-        <v>33</v>
-      </c>
-      <c r="F26" s="44" t="s">
-        <v>59</v>
-      </c>
-      <c r="G26" s="55" t="s">
+      <c r="E27" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="F27" s="56" t="s">
+        <v>20</v>
+      </c>
+      <c r="G27" s="57" t="s">
+        <v>94</v>
+      </c>
+      <c r="H27" s="76" t="s">
+        <v>112</v>
+      </c>
+      <c r="I27" s="53" t="s">
+        <v>129</v>
+      </c>
+      <c r="J27"/>
+      <c r="K27"/>
+      <c r="L27"/>
+      <c r="M27"/>
+      <c r="N27"/>
+      <c r="O27"/>
+      <c r="P27"/>
+      <c r="Q27"/>
+      <c r="R27"/>
+      <c r="S27"/>
+      <c r="T27"/>
+      <c r="U27"/>
+      <c r="V27"/>
+      <c r="W27"/>
+      <c r="X27"/>
+      <c r="Y27"/>
+      <c r="Z27"/>
+      <c r="AA27"/>
+      <c r="AB27"/>
+      <c r="AC27"/>
+    </row>
+    <row r="28" spans="1:29" ht="28.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="89" t="s">
+        <v>34</v>
+      </c>
+      <c r="B28" s="43" t="s">
         <v>97</v>
       </c>
-      <c r="H26" s="47" t="s">
-        <v>78</v>
-      </c>
-      <c r="I26" s="48"/>
-      <c r="J26"/>
-      <c r="K26"/>
-      <c r="L26"/>
-      <c r="M26"/>
-      <c r="N26"/>
-      <c r="O26"/>
-      <c r="P26"/>
-      <c r="Q26"/>
-      <c r="R26"/>
-      <c r="S26"/>
-      <c r="T26"/>
-      <c r="U26"/>
-      <c r="V26"/>
-      <c r="W26"/>
-      <c r="X26"/>
-      <c r="Y26"/>
-      <c r="Z26"/>
-      <c r="AA26"/>
-      <c r="AB26"/>
-      <c r="AC26"/>
-    </row>
-    <row r="27" spans="1:29" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="109"/>
-      <c r="B27" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C27" s="11" t="s">
+      <c r="C28" s="43" t="s">
+        <v>102</v>
+      </c>
+      <c r="D28" s="43" t="s">
+        <v>19</v>
+      </c>
+      <c r="E28" s="44" t="s">
+        <v>32</v>
+      </c>
+      <c r="F28" s="45" t="s">
+        <v>20</v>
+      </c>
+      <c r="G28" s="46" t="s">
+        <v>93</v>
+      </c>
+      <c r="H28" s="69" t="s">
         <v>112</v>
       </c>
-      <c r="D27" s="11" t="s">
+      <c r="I28" s="48" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="29" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="90"/>
+      <c r="B29" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="D29" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="E29" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="F29" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F27" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="G27" s="56" t="s">
-        <v>97</v>
-      </c>
-      <c r="H27" s="77" t="s">
-        <v>114</v>
-      </c>
-      <c r="I27" s="19"/>
-    </row>
-    <row r="28" spans="1:29" s="17" customFormat="1" ht="55.5" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="110"/>
-      <c r="B28" s="50" t="s">
-        <v>57</v>
-      </c>
-      <c r="C28" s="50" t="s">
-        <v>62</v>
-      </c>
-      <c r="D28" s="50" t="s">
-        <v>19</v>
-      </c>
-      <c r="E28" s="51" t="s">
-        <v>33</v>
-      </c>
-      <c r="F28" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="G28" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="H28" s="78" t="s">
-        <v>114</v>
-      </c>
-      <c r="I28" s="54" t="s">
-        <v>131</v>
-      </c>
-      <c r="J28"/>
-      <c r="K28"/>
-      <c r="L28"/>
-      <c r="M28"/>
-      <c r="N28"/>
-      <c r="O28"/>
-      <c r="P28"/>
-      <c r="Q28"/>
-      <c r="R28"/>
-      <c r="S28"/>
-      <c r="T28"/>
-      <c r="U28"/>
-      <c r="V28"/>
-      <c r="W28"/>
-      <c r="X28"/>
-      <c r="Y28"/>
-      <c r="Z28"/>
-      <c r="AA28"/>
-      <c r="AB28"/>
-      <c r="AC28"/>
-    </row>
-    <row r="29" spans="1:29" ht="28.5" hidden="1" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="91" t="s">
-        <v>35</v>
-      </c>
-      <c r="B29" s="43" t="s">
+      <c r="G29" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="H29" s="75" t="s">
+        <v>112</v>
+      </c>
+      <c r="I29" s="19"/>
+    </row>
+    <row r="30" spans="1:29" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="90"/>
+      <c r="B30" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="C29" s="43" t="s">
-        <v>104</v>
-      </c>
-      <c r="D29" s="43" t="s">
-        <v>19</v>
-      </c>
-      <c r="E29" s="44" t="s">
-        <v>33</v>
-      </c>
-      <c r="F29" s="45" t="s">
-        <v>20</v>
-      </c>
-      <c r="G29" s="46" t="s">
-        <v>94</v>
-      </c>
-      <c r="H29" s="71" t="s">
-        <v>114</v>
-      </c>
-      <c r="I29" s="48" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="30" spans="1:29" ht="25.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="92"/>
-      <c r="B30" s="11" t="s">
+      <c r="C30" s="11" t="s">
         <v>100</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>103</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E30" s="36" t="s">
-        <v>33</v>
+      <c r="E30" s="10" t="s">
+        <v>20</v>
       </c>
       <c r="F30" s="10" t="s">
         <v>20</v>
       </c>
       <c r="G30" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="H30" s="49" t="s">
-        <v>78</v>
+        <v>93</v>
+      </c>
+      <c r="H30" s="75" t="s">
+        <v>77</v>
       </c>
       <c r="I30" s="19"/>
     </row>
-    <row r="31" spans="1:29" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="92"/>
+    <row r="31" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="90"/>
       <c r="B31" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E31" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F31" s="10" t="s">
-        <v>20</v>
+      <c r="E31" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="F31" s="11" t="s">
+        <v>143</v>
       </c>
       <c r="G31" s="37" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H31" s="49" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I31" s="19"/>
     </row>
-    <row r="32" spans="1:29" ht="25.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="92"/>
+    <row r="32" spans="1:29" s="16" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="90"/>
       <c r="B32" s="11" t="s">
-        <v>105</v>
+        <v>54</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="D32" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E32" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="F32" s="11" t="s">
-        <v>59</v>
+      <c r="E32" s="36" t="s">
+        <v>32</v>
+      </c>
+      <c r="F32" s="36" t="s">
+        <v>143</v>
       </c>
       <c r="G32" s="37" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H32" s="49" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I32" s="19"/>
-    </row>
-    <row r="33" spans="1:29" s="16" customFormat="1" ht="37.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="92"/>
+      <c r="J32"/>
+      <c r="K32"/>
+      <c r="L32"/>
+      <c r="M32"/>
+      <c r="N32"/>
+      <c r="O32"/>
+      <c r="P32"/>
+      <c r="Q32"/>
+      <c r="R32"/>
+      <c r="S32"/>
+      <c r="T32"/>
+      <c r="U32"/>
+      <c r="V32"/>
+      <c r="W32"/>
+      <c r="X32"/>
+      <c r="Y32"/>
+      <c r="Z32"/>
+      <c r="AA32"/>
+      <c r="AB32"/>
+      <c r="AC32"/>
+    </row>
+    <row r="33" spans="1:29" s="16" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="90"/>
       <c r="B33" s="11" t="s">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>90</v>
+        <v>134</v>
       </c>
       <c r="D33" s="11" t="s">
         <v>19</v>
       </c>
       <c r="E33" s="36" t="s">
-        <v>33</v>
-      </c>
-      <c r="F33" s="36" t="s">
         <v>20</v>
       </c>
+      <c r="F33" s="11" t="s">
+        <v>58</v>
+      </c>
       <c r="G33" s="37" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H33" s="49" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I33" s="19"/>
       <c r="J33"/>
@@ -2915,30 +2944,32 @@
       <c r="AB33"/>
       <c r="AC33"/>
     </row>
-    <row r="34" spans="1:29" s="16" customFormat="1" ht="37.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="92"/>
+    <row r="34" spans="1:29" s="16" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="90"/>
       <c r="B34" s="11" t="s">
-        <v>26</v>
+        <v>137</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>19</v>
       </c>
       <c r="E34" s="36" t="s">
-        <v>20</v>
-      </c>
-      <c r="F34" s="11" t="s">
         <v>59</v>
       </c>
+      <c r="F34" s="36" t="s">
+        <v>59</v>
+      </c>
       <c r="G34" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="H34" s="49" t="s">
-        <v>78</v>
-      </c>
-      <c r="I34" s="19"/>
+        <v>93</v>
+      </c>
+      <c r="H34" s="75" t="s">
+        <v>112</v>
+      </c>
+      <c r="I34" s="19" t="s">
+        <v>139</v>
+      </c>
       <c r="J34"/>
       <c r="K34"/>
       <c r="L34"/>
@@ -2960,32 +2991,30 @@
       <c r="AB34"/>
       <c r="AC34"/>
     </row>
-    <row r="35" spans="1:29" s="16" customFormat="1" ht="37.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="92"/>
+    <row r="35" spans="1:29" s="16" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="90"/>
       <c r="B35" s="11" t="s">
-        <v>139</v>
+        <v>105</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>140</v>
+        <v>106</v>
       </c>
       <c r="D35" s="11" t="s">
         <v>19</v>
       </c>
       <c r="E35" s="36" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="F35" s="36" t="s">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="G35" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="H35" s="77" t="s">
-        <v>114</v>
-      </c>
-      <c r="I35" s="19" t="s">
-        <v>141</v>
-      </c>
+        <v>93</v>
+      </c>
+      <c r="H35" s="75" t="s">
+        <v>112</v>
+      </c>
+      <c r="I35" s="19"/>
       <c r="J35"/>
       <c r="K35"/>
       <c r="L35"/>
@@ -3007,30 +3036,30 @@
       <c r="AB35"/>
       <c r="AC35"/>
     </row>
-    <row r="36" spans="1:29" s="16" customFormat="1" ht="33.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="92"/>
-      <c r="B36" s="11" t="s">
+    <row r="36" spans="1:29" s="16" customFormat="1" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="91"/>
+      <c r="B36" s="50" t="s">
         <v>107</v>
       </c>
-      <c r="C36" s="11" t="s">
+      <c r="C36" s="50" t="s">
         <v>108</v>
       </c>
-      <c r="D36" s="11" t="s">
+      <c r="D36" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="E36" s="36" t="s">
-        <v>33</v>
-      </c>
-      <c r="F36" s="36" t="s">
+      <c r="E36" s="51" t="s">
+        <v>32</v>
+      </c>
+      <c r="F36" s="51" t="s">
         <v>20</v>
       </c>
-      <c r="G36" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="H36" s="49" t="s">
-        <v>78</v>
-      </c>
-      <c r="I36" s="19"/>
+      <c r="G36" s="52" t="s">
+        <v>93</v>
+      </c>
+      <c r="H36" s="76" t="s">
+        <v>112</v>
+      </c>
+      <c r="I36" s="53"/>
       <c r="J36"/>
       <c r="K36"/>
       <c r="L36"/>
@@ -3052,71 +3081,21 @@
       <c r="AB36"/>
       <c r="AC36"/>
     </row>
-    <row r="37" spans="1:29" s="16" customFormat="1" ht="33.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="93"/>
-      <c r="B37" s="50" t="s">
-        <v>109</v>
-      </c>
-      <c r="C37" s="50" t="s">
-        <v>110</v>
-      </c>
-      <c r="D37" s="50" t="s">
-        <v>19</v>
-      </c>
-      <c r="E37" s="51" t="s">
-        <v>33</v>
-      </c>
-      <c r="F37" s="51" t="s">
-        <v>20</v>
-      </c>
-      <c r="G37" s="52" t="s">
-        <v>94</v>
-      </c>
-      <c r="H37" s="53" t="s">
-        <v>78</v>
-      </c>
-      <c r="I37" s="54"/>
-      <c r="J37"/>
-      <c r="K37"/>
-      <c r="L37"/>
-      <c r="M37"/>
-      <c r="N37"/>
-      <c r="O37"/>
-      <c r="P37"/>
-      <c r="Q37"/>
-      <c r="R37"/>
-      <c r="S37"/>
-      <c r="T37"/>
-      <c r="U37"/>
-      <c r="V37"/>
-      <c r="W37"/>
-      <c r="X37"/>
-      <c r="Y37"/>
-      <c r="Z37"/>
-      <c r="AA37"/>
-      <c r="AB37"/>
-      <c r="AC37"/>
-    </row>
+    <row r="37" spans="1:29" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="G5:G37" xr:uid="{4AB4A1F4-D2AB-4474-B05F-C8B13F4E557C}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Nathen Reed"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="G5:G36" xr:uid="{4AB4A1F4-D2AB-4474-B05F-C8B13F4E557C}"/>
   <mergeCells count="11">
-    <mergeCell ref="A29:A37"/>
-    <mergeCell ref="A13:A15"/>
-    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="A28:A36"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="A10:A11"/>
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="B4:I4"/>
-    <mergeCell ref="A26:A28"/>
+    <mergeCell ref="A25:A27"/>
     <mergeCell ref="A6:A8"/>
-    <mergeCell ref="A16:A18"/>
-    <mergeCell ref="A19:A25"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A18:A24"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B4" r:id="rId1" xr:uid="{73359DB6-C291-4AB2-82A3-BE2171E1A73F}"/>
@@ -3142,28 +3121,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="115" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="118"/>
-      <c r="C1" s="118"/>
-      <c r="D1" s="118"/>
-      <c r="E1" s="118"/>
-      <c r="F1" s="118"/>
-      <c r="G1" s="81"/>
+      <c r="B1" s="116"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="79"/>
     </row>
     <row r="2" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="39" t="s">
-        <v>83</v>
-      </c>
-      <c r="B2" s="119" t="s">
-        <v>86</v>
-      </c>
-      <c r="C2" s="120"/>
-      <c r="D2" s="120"/>
-      <c r="E2" s="120"/>
-      <c r="F2" s="120"/>
-      <c r="G2" s="82"/>
+        <v>82</v>
+      </c>
+      <c r="B2" s="117" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" s="118"/>
+      <c r="D2" s="118"/>
+      <c r="E2" s="118"/>
+      <c r="F2" s="118"/>
+      <c r="G2" s="80"/>
     </row>
     <row r="3" spans="1:8" s="26" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
@@ -3181,223 +3160,223 @@
       <c r="E3" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="79" t="s">
+      <c r="F3" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="83" t="s">
-        <v>88</v>
-      </c>
-      <c r="H3" s="80"/>
+      <c r="G3" s="81" t="s">
+        <v>87</v>
+      </c>
+      <c r="H3" s="78"/>
     </row>
     <row r="4" spans="1:8" ht="225.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="84" t="s">
+      <c r="A4" s="82" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="84" t="s">
-        <v>87</v>
-      </c>
-      <c r="C4" s="85" t="s">
+      <c r="B4" s="82" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" s="83" t="s">
+        <v>122</v>
+      </c>
+      <c r="D4" s="82" t="s">
+        <v>123</v>
+      </c>
+      <c r="E4" s="82" t="s">
         <v>124</v>
       </c>
-      <c r="D4" s="84" t="s">
+      <c r="F4" s="82" t="s">
         <v>125</v>
       </c>
-      <c r="E4" s="84" t="s">
+      <c r="G4" s="82" t="s">
         <v>126</v>
       </c>
-      <c r="F4" s="84" t="s">
-        <v>127</v>
-      </c>
-      <c r="G4" s="84" t="s">
-        <v>128</v>
-      </c>
     </row>
     <row r="5" spans="1:8" ht="143.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="84" t="s">
+      <c r="A5" s="82" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="82" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="84" t="s">
+      <c r="C5" s="83" t="s">
+        <v>84</v>
+      </c>
+      <c r="D5" s="82" t="s">
+        <v>130</v>
+      </c>
+      <c r="E5" s="82" t="s">
+        <v>131</v>
+      </c>
+      <c r="F5" s="82" t="s">
+        <v>132</v>
+      </c>
+      <c r="G5" s="82" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="191.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="82" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="85" t="s">
-        <v>85</v>
-      </c>
-      <c r="D5" s="84" t="s">
-        <v>132</v>
-      </c>
-      <c r="E5" s="84" t="s">
-        <v>133</v>
-      </c>
-      <c r="F5" s="84" t="s">
-        <v>134</v>
-      </c>
-      <c r="G5" s="84" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="191.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="84" t="s">
+      <c r="B6" s="82" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="84" t="s">
+      <c r="C6" s="83" t="s">
+        <v>84</v>
+      </c>
+      <c r="D6" s="82"/>
+      <c r="E6" s="82"/>
+      <c r="F6" s="82"/>
+      <c r="G6" s="82"/>
+    </row>
+    <row r="7" spans="1:8" ht="115.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="82" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="82" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="83" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" s="82"/>
+      <c r="E7" s="82"/>
+      <c r="F7" s="82"/>
+      <c r="G7" s="82"/>
+    </row>
+    <row r="8" spans="1:8" s="29" customFormat="1" ht="227.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="84" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="119" t="s">
         <v>66</v>
       </c>
-      <c r="C6" s="85" t="s">
-        <v>85</v>
-      </c>
-      <c r="D6" s="84"/>
-      <c r="E6" s="84"/>
-      <c r="F6" s="84"/>
-      <c r="G6" s="84"/>
-    </row>
-    <row r="7" spans="1:8" ht="115.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="84" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="84" t="s">
-        <v>73</v>
-      </c>
-      <c r="C7" s="85" t="s">
-        <v>85</v>
-      </c>
-      <c r="D7" s="84"/>
-      <c r="E7" s="84"/>
-      <c r="F7" s="84"/>
-      <c r="G7" s="84"/>
-    </row>
-    <row r="8" spans="1:8" s="29" customFormat="1" ht="227.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="86" t="s">
-        <v>72</v>
-      </c>
-      <c r="B8" s="121" t="s">
+      <c r="C8" s="83" t="s">
+        <v>84</v>
+      </c>
+      <c r="D8" s="82"/>
+      <c r="E8" s="85"/>
+      <c r="F8" s="82"/>
+      <c r="G8" s="82"/>
+    </row>
+    <row r="9" spans="1:8" ht="238.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="82" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="85" t="s">
-        <v>85</v>
-      </c>
-      <c r="D8" s="84"/>
-      <c r="E8" s="87"/>
-      <c r="F8" s="84"/>
-      <c r="G8" s="84"/>
-    </row>
-    <row r="9" spans="1:8" ht="238.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="84" t="s">
+      <c r="B9" s="119"/>
+      <c r="C9" s="83" t="s">
+        <v>84</v>
+      </c>
+      <c r="D9" s="82"/>
+      <c r="E9" s="85"/>
+      <c r="F9" s="82"/>
+      <c r="G9" s="82"/>
+    </row>
+    <row r="10" spans="1:8" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="86" t="s">
         <v>68</v>
       </c>
-      <c r="B9" s="121"/>
-      <c r="C9" s="85" t="s">
-        <v>85</v>
-      </c>
-      <c r="D9" s="84"/>
-      <c r="E9" s="87"/>
-      <c r="F9" s="84"/>
-      <c r="G9" s="84"/>
-    </row>
-    <row r="10" spans="1:8" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="88" t="s">
+      <c r="B10" s="119"/>
+      <c r="C10" s="86" t="s">
+        <v>84</v>
+      </c>
+      <c r="D10" s="86"/>
+      <c r="E10" s="85"/>
+      <c r="F10" s="82"/>
+      <c r="G10" s="82"/>
+    </row>
+    <row r="11" spans="1:8" ht="145.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="82" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="121"/>
-      <c r="C10" s="88" t="s">
-        <v>85</v>
-      </c>
-      <c r="D10" s="88"/>
-      <c r="E10" s="87"/>
-      <c r="F10" s="84"/>
-      <c r="G10" s="84"/>
-    </row>
-    <row r="11" spans="1:8" ht="145.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="84" t="s">
+      <c r="B11" s="119"/>
+      <c r="C11" s="83" t="s">
+        <v>84</v>
+      </c>
+      <c r="D11" s="82"/>
+      <c r="E11" s="85"/>
+      <c r="F11" s="82"/>
+      <c r="G11" s="82"/>
+    </row>
+    <row r="12" spans="1:8" s="30" customFormat="1" ht="102" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="82" t="s">
         <v>70</v>
       </c>
-      <c r="B11" s="121"/>
-      <c r="C11" s="85" t="s">
-        <v>85</v>
-      </c>
-      <c r="D11" s="84"/>
-      <c r="E11" s="87"/>
-      <c r="F11" s="84"/>
-      <c r="G11" s="84"/>
-    </row>
-    <row r="12" spans="1:8" s="30" customFormat="1" ht="102" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="84" t="s">
-        <v>71</v>
-      </c>
-      <c r="B12" s="121"/>
-      <c r="C12" s="85" t="s">
-        <v>85</v>
-      </c>
-      <c r="D12" s="84"/>
-      <c r="E12" s="87"/>
-      <c r="F12" s="84"/>
-      <c r="G12" s="84"/>
+      <c r="B12" s="119"/>
+      <c r="C12" s="83" t="s">
+        <v>84</v>
+      </c>
+      <c r="D12" s="82"/>
+      <c r="E12" s="85"/>
+      <c r="F12" s="82"/>
+      <c r="G12" s="82"/>
     </row>
     <row r="13" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="84" t="s">
+      <c r="A13" s="82" t="s">
+        <v>114</v>
+      </c>
+      <c r="B13" s="82" t="s">
+        <v>117</v>
+      </c>
+      <c r="C13" s="83" t="s">
+        <v>84</v>
+      </c>
+      <c r="D13" s="82"/>
+      <c r="E13" s="82"/>
+      <c r="F13" s="82"/>
+      <c r="G13" s="82"/>
+    </row>
+    <row r="14" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="82" t="s">
+        <v>115</v>
+      </c>
+      <c r="B14" s="82" t="s">
+        <v>118</v>
+      </c>
+      <c r="C14" s="83" t="s">
+        <v>84</v>
+      </c>
+      <c r="D14" s="82"/>
+      <c r="E14" s="82"/>
+      <c r="F14" s="82"/>
+      <c r="G14" s="82"/>
+    </row>
+    <row r="15" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="82" t="s">
         <v>116</v>
       </c>
-      <c r="B13" s="84" t="s">
+      <c r="B15" s="82" t="s">
         <v>119</v>
       </c>
-      <c r="C13" s="85" t="s">
-        <v>85</v>
-      </c>
-      <c r="D13" s="84"/>
-      <c r="E13" s="84"/>
-      <c r="F13" s="84"/>
-      <c r="G13" s="84"/>
-    </row>
-    <row r="14" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="84" t="s">
-        <v>117</v>
-      </c>
-      <c r="B14" s="84" t="s">
+      <c r="C15" s="83" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="82"/>
+      <c r="E15" s="82"/>
+      <c r="F15" s="82"/>
+      <c r="G15" s="82"/>
+    </row>
+    <row r="16" spans="1:8" ht="84" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="82" t="s">
         <v>120</v>
       </c>
-      <c r="C14" s="85" t="s">
-        <v>85</v>
-      </c>
-      <c r="D14" s="84"/>
-      <c r="E14" s="84"/>
-      <c r="F14" s="84"/>
-      <c r="G14" s="84"/>
-    </row>
-    <row r="15" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="84" t="s">
-        <v>118</v>
-      </c>
-      <c r="B15" s="84" t="s">
+      <c r="B16" s="82" t="s">
         <v>121</v>
       </c>
-      <c r="C15" s="85" t="s">
-        <v>85</v>
-      </c>
-      <c r="D15" s="84"/>
-      <c r="E15" s="84"/>
-      <c r="F15" s="84"/>
-      <c r="G15" s="84"/>
-    </row>
-    <row r="16" spans="1:8" ht="84" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="84" t="s">
-        <v>122</v>
-      </c>
-      <c r="B16" s="84" t="s">
-        <v>123</v>
-      </c>
-      <c r="C16" s="84"/>
-      <c r="D16" s="84"/>
-      <c r="E16" s="84"/>
-      <c r="F16" s="84"/>
-      <c r="G16" s="84"/>
+      <c r="C16" s="82"/>
+      <c r="D16" s="82"/>
+      <c r="E16" s="82"/>
+      <c r="F16" s="82"/>
+      <c r="G16" s="82"/>
     </row>
     <row r="17" spans="1:7" ht="99.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="84"/>
-      <c r="B17" s="84"/>
-      <c r="C17" s="84"/>
-      <c r="D17" s="84"/>
-      <c r="E17" s="84"/>
-      <c r="F17" s="84"/>
-      <c r="G17" s="84"/>
+      <c r="A17" s="82"/>
+      <c r="B17" s="82"/>
+      <c r="C17" s="82"/>
+      <c r="D17" s="82"/>
+      <c r="E17" s="82"/>
+      <c r="F17" s="82"/>
+      <c r="G17" s="82"/>
     </row>
     <row r="18" spans="1:7" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="21"/>
@@ -3774,15 +3753,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="ff8a4b2e-b0c8-4039-a689-d1a7f36f4382">
@@ -3792,6 +3762,15 @@
     <Notes xmlns="ff8a4b2e-b0c8-4039-a689-d1a7f36f4382" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3814,14 +3793,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8F3069D-89E7-4007-93BF-1DB2942FF756}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76F271AB-EFB2-4823-A2F0-9F2289E658DB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3832,4 +3803,12 @@
     <ds:schemaRef ds:uri="f716dd8a-49a0-4c40-b209-038e1651b548"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8F3069D-89E7-4007-93BF-1DB2942FF756}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added boss wolf class, spawner, Health Widget.
</commit_message>
<xml_diff>
--- a/Red Team Tracebility and Testing.xlsx
+++ b/Red Team Tracebility and Testing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Program Files\Epic Games\UE_5.7\redteam\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4472431A-0CCB-4D31-AD20-F02E702BD0A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B16AD1-5BC3-4351-8C27-F1E2C2FCC003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{19EF330C-6F54-4365-A47E-10806019DE9B}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="165">
   <si>
     <t>Prototype Title:</t>
   </si>
@@ -296,28 +296,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> Ranged Attack</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Boss</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t xml:space="preserve"> Movement</t>
     </r>
   </si>
@@ -347,24 +325,15 @@
     <t>Boss Class</t>
   </si>
   <si>
-    <t>Use health widgets to visibly show player health changes, made more legible using segments.</t>
-  </si>
-  <si>
     <t>Display the boss health over the boss.</t>
   </si>
   <si>
     <t>Boss is defeated after health reaches zero.</t>
   </si>
   <si>
-    <t>Create a health system for the boss. They lose health only after they finish charging</t>
-  </si>
-  <si>
     <t>Enemies should be destroyed when hit by player</t>
   </si>
   <si>
-    <t>N</t>
-  </si>
-  <si>
     <t>Jump Attack</t>
   </si>
   <si>
@@ -569,9 +538,6 @@
     <t>Checkpoint Updated With custom FB. -Nathen Reed</t>
   </si>
   <si>
-    <t>Created levels 1 and 2 pending final third level. -Nathen Reed</t>
-  </si>
-  <si>
     <t>Added simple moving platform that ping pongs between two spots. -Nathen Reed</t>
   </si>
   <si>
@@ -579,6 +545,66 @@
   </si>
   <si>
     <t>Added but needs som small adjustments to projectile.</t>
+  </si>
+  <si>
+    <t>Added but may be hidden in final version to fit style</t>
+  </si>
+  <si>
+    <t>added, requires a win screen post win.</t>
+  </si>
+  <si>
+    <t>Create a health system for the boss. They lose health but get a shield briefly after taking a hit.</t>
+  </si>
+  <si>
+    <t>Shield works, may need a bit of tweaking to fling the player on each hit to prevent them from hitting the boss over and over.</t>
+  </si>
+  <si>
+    <t>Added but not currently used any longer as collectables didn’t fit as well.</t>
+  </si>
+  <si>
+    <t>enemy turning invisible</t>
+  </si>
+  <si>
+    <t>sometimes enemy would turn invisibile</t>
+  </si>
+  <si>
+    <t>Was just a missing flipbook designation.</t>
+  </si>
+  <si>
+    <t>Nathen Reed (5:39PM, 6/14/2026)</t>
+  </si>
+  <si>
+    <t>Player health should tick down upon taking damage displayed with a widget or UI Element.</t>
+  </si>
+  <si>
+    <t>Player getting blocked by the overlap zone for the stomp attack instead of overlapping and bouncing.</t>
+  </si>
+  <si>
+    <t>issues with overlapping player and stomp zone</t>
+  </si>
+  <si>
+    <t>Addded a Slight delay before knockback was applied, and adjusted some of the logic for the hitbox.</t>
+  </si>
+  <si>
+    <t>Boss would randomly stop or keep going.</t>
+  </si>
+  <si>
+    <t>during charage attack the boss wouldn’t halt or would start moving faster without pausing movement.</t>
+  </si>
+  <si>
+    <t>Fixed by adjusting booleans to record current state more accurately with branches in the movement controls. As well the attack box was clipping the ground slightly due causing it to end charge early.</t>
+  </si>
+  <si>
+    <t>charge wouldn’t fling and damage the player immediately.</t>
+  </si>
+  <si>
+    <t>during charge the boss would keep bumping into the player instead of flinging them.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Increased knockback force and extended the attack zone further. </t>
+  </si>
+  <si>
+    <t>Created levels 1 and 2, Final/boss level added by Hunter Eck. -Nathen Reed</t>
   </si>
 </sst>
 </file>
@@ -776,12 +802,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -801,6 +821,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1273,7 +1299,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1367,7 +1393,7 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1376,9 +1402,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1390,45 +1414,43 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="28" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="13" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1441,11 +1463,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1494,16 +1516,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1595,6 +1614,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1932,30 +1963,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="98" t="s">
-        <v>81</v>
-      </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
+      <c r="A1" s="93" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="94"/>
+      <c r="C1" s="94"/>
+      <c r="D1" s="94"/>
+      <c r="E1" s="94"/>
+      <c r="F1" s="94"/>
+      <c r="G1" s="94"/>
+      <c r="H1" s="94"/>
+      <c r="I1" s="94"/>
     </row>
     <row r="2" spans="1:29" s="3" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="95"/>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="96"/>
-      <c r="H2" s="96"/>
-      <c r="I2" s="97"/>
+      <c r="B2" s="90"/>
+      <c r="C2" s="91"/>
+      <c r="D2" s="91"/>
+      <c r="E2" s="91"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="91"/>
+      <c r="H2" s="91"/>
+      <c r="I2" s="92"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
@@ -1974,88 +2005,88 @@
       <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="100" t="s">
-        <v>83</v>
-      </c>
-      <c r="C3" s="101"/>
-      <c r="D3" s="101"/>
-      <c r="E3" s="101"/>
-      <c r="F3" s="101"/>
-      <c r="G3" s="101"/>
-      <c r="H3" s="101"/>
-      <c r="I3" s="102"/>
+      <c r="B3" s="95" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="96"/>
+      <c r="G3" s="96"/>
+      <c r="H3" s="96"/>
+      <c r="I3" s="97"/>
     </row>
     <row r="4" spans="1:29" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="38" t="s">
-        <v>82</v>
-      </c>
-      <c r="B4" s="103" t="s">
-        <v>85</v>
-      </c>
-      <c r="C4" s="104"/>
-      <c r="D4" s="104"/>
-      <c r="E4" s="104"/>
-      <c r="F4" s="104"/>
-      <c r="G4" s="104"/>
-      <c r="H4" s="104"/>
-      <c r="I4" s="105"/>
+        <v>78</v>
+      </c>
+      <c r="B4" s="98" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="99"/>
+      <c r="D4" s="99"/>
+      <c r="E4" s="99"/>
+      <c r="F4" s="99"/>
+      <c r="G4" s="99"/>
+      <c r="H4" s="99"/>
+      <c r="I4" s="100"/>
     </row>
     <row r="5" spans="1:29" s="2" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="61" t="s">
+      <c r="A5" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="61" t="s">
+      <c r="B5" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="61" t="s">
+      <c r="C5" s="57" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="61" t="s">
+      <c r="D5" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="61" t="s">
+      <c r="E5" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="61" t="s">
+      <c r="F5" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="61" t="s">
+      <c r="G5" s="57" t="s">
         <v>15</v>
       </c>
       <c r="H5" s="35" t="s">
         <v>57</v>
       </c>
       <c r="I5" s="35" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:29" s="8" customFormat="1" ht="46.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="109" t="s">
+      <c r="A6" s="104" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="63" t="s">
+      <c r="B6" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="64" t="s">
-        <v>80</v>
-      </c>
-      <c r="D6" s="64" t="s">
+      <c r="C6" s="60" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="44" t="s">
+      <c r="E6" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="45" t="s">
+      <c r="F6" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="G6" s="65" t="s">
-        <v>94</v>
-      </c>
-      <c r="H6" s="69" t="s">
-        <v>112</v>
-      </c>
-      <c r="I6" s="70" t="s">
-        <v>113</v>
+      <c r="G6" s="61" t="s">
+        <v>90</v>
+      </c>
+      <c r="H6" s="65" t="s">
+        <v>108</v>
+      </c>
+      <c r="I6" s="66" t="s">
+        <v>109</v>
       </c>
       <c r="J6" s="20"/>
       <c r="K6"/>
@@ -2079,8 +2110,8 @@
       <c r="AC6"/>
     </row>
     <row r="7" spans="1:29" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="110"/>
-      <c r="B7" s="66" t="s">
+      <c r="A7" s="105"/>
+      <c r="B7" s="62" t="s">
         <v>50</v>
       </c>
       <c r="C7" s="9" t="s">
@@ -2090,47 +2121,47 @@
         <v>19</v>
       </c>
       <c r="E7" s="36" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F7" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G7" s="67" t="s">
-        <v>94</v>
-      </c>
-      <c r="H7" s="75" t="s">
-        <v>112</v>
-      </c>
-      <c r="I7" s="87" t="s">
-        <v>136</v>
+      <c r="G7" s="63" t="s">
+        <v>90</v>
+      </c>
+      <c r="H7" s="71" t="s">
+        <v>108</v>
+      </c>
+      <c r="I7" s="82" t="s">
+        <v>132</v>
       </c>
       <c r="J7" s="20"/>
     </row>
     <row r="8" spans="1:29" s="7" customFormat="1" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="111"/>
-      <c r="B8" s="50" t="s">
+      <c r="A8" s="106"/>
+      <c r="B8" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="50" t="s">
+      <c r="C8" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="68" t="s">
+      <c r="D8" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="51" t="s">
+      <c r="E8" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="51" t="s">
+      <c r="F8" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="57" t="s">
-        <v>94</v>
-      </c>
-      <c r="H8" s="76" t="s">
-        <v>112</v>
-      </c>
-      <c r="I8" s="53" t="s">
-        <v>148</v>
+      <c r="G8" s="53" t="s">
+        <v>90</v>
+      </c>
+      <c r="H8" s="72" t="s">
+        <v>108</v>
+      </c>
+      <c r="I8" s="49" t="s">
+        <v>143</v>
       </c>
       <c r="J8" s="20"/>
       <c r="K8"/>
@@ -2154,14 +2185,14 @@
       <c r="AC8"/>
     </row>
     <row r="9" spans="1:29" ht="40.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="62" t="s">
+      <c r="A9" s="58" t="s">
         <v>21</v>
       </c>
       <c r="B9" s="31" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C9" s="32" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D9" s="33" t="s">
         <v>19</v>
@@ -2172,53 +2203,53 @@
       <c r="F9" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="G9" s="42" t="s">
-        <v>94</v>
-      </c>
-      <c r="H9" s="73" t="s">
-        <v>112</v>
-      </c>
-      <c r="I9" s="74" t="s">
-        <v>135</v>
+      <c r="G9" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="H9" s="69" t="s">
+        <v>108</v>
+      </c>
+      <c r="I9" s="70" t="s">
+        <v>131</v>
       </c>
       <c r="J9" s="20"/>
     </row>
     <row r="10" spans="1:29" ht="42" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="93" t="s">
+      <c r="A10" s="88" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="43" t="s">
+      <c r="B10" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="43" t="s">
+      <c r="C10" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="64" t="s">
+      <c r="D10" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="44" t="s">
+      <c r="E10" s="42" t="s">
         <v>59</v>
       </c>
-      <c r="F10" s="44" t="s">
+      <c r="F10" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="G10" s="54" t="s">
-        <v>96</v>
-      </c>
-      <c r="H10" s="69" t="s">
-        <v>112</v>
-      </c>
-      <c r="I10" s="48" t="s">
-        <v>127</v>
+      <c r="G10" s="50" t="s">
+        <v>92</v>
+      </c>
+      <c r="H10" s="65" t="s">
+        <v>108</v>
+      </c>
+      <c r="I10" s="45" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:29" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="94"/>
+      <c r="A11" s="89"/>
       <c r="B11" s="32" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C11" s="32" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D11" s="33" t="s">
         <v>19</v>
@@ -2229,48 +2260,48 @@
       <c r="F11" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="G11" s="88" t="s">
-        <v>96</v>
-      </c>
-      <c r="H11" s="73" t="s">
-        <v>112</v>
-      </c>
-      <c r="I11" s="74" t="s">
-        <v>144</v>
+      <c r="G11" s="83" t="s">
+        <v>92</v>
+      </c>
+      <c r="H11" s="69" t="s">
+        <v>108</v>
+      </c>
+      <c r="I11" s="70" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:29" ht="51.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="92" t="s">
-        <v>111</v>
-      </c>
-      <c r="B12" s="43" t="s">
+      <c r="A12" s="87" t="s">
+        <v>107</v>
+      </c>
+      <c r="B12" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="43" t="s">
+      <c r="C12" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="43" t="s">
+      <c r="D12" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="44" t="s">
+      <c r="E12" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="F12" s="45" t="s">
+      <c r="F12" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="G12" s="54" t="s">
-        <v>96</v>
-      </c>
-      <c r="H12" s="69" t="s">
-        <v>112</v>
-      </c>
-      <c r="I12" s="48" t="s">
-        <v>145</v>
+      <c r="G12" s="50" t="s">
+        <v>92</v>
+      </c>
+      <c r="H12" s="65" t="s">
+        <v>108</v>
+      </c>
+      <c r="I12" s="45" t="s">
+        <v>141</v>
       </c>
       <c r="J12" s="20"/>
     </row>
     <row r="13" spans="1:29" ht="51" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="90"/>
+      <c r="A13" s="85"/>
       <c r="B13" s="11" t="s">
         <v>29</v>
       </c>
@@ -2286,121 +2317,127 @@
       <c r="F13" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="G13" s="55" t="s">
-        <v>96</v>
-      </c>
-      <c r="H13" s="69" t="s">
-        <v>112</v>
+      <c r="G13" s="51" t="s">
+        <v>92</v>
+      </c>
+      <c r="H13" s="65" t="s">
+        <v>108</v>
       </c>
       <c r="I13" s="19" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="J13" s="20"/>
     </row>
     <row r="14" spans="1:29" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="91"/>
-      <c r="B14" s="50" t="s">
+      <c r="A14" s="86"/>
+      <c r="B14" s="46" t="s">
+        <v>87</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="52" t="s">
+        <v>58</v>
+      </c>
+      <c r="G14" s="56" t="s">
         <v>91</v>
       </c>
-      <c r="C14" s="50" t="s">
-        <v>92</v>
-      </c>
-      <c r="D14" s="50" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="51" t="s">
-        <v>20</v>
-      </c>
-      <c r="F14" s="56" t="s">
-        <v>58</v>
-      </c>
-      <c r="G14" s="60" t="s">
-        <v>95</v>
-      </c>
-      <c r="H14" s="76" t="s">
-        <v>112</v>
-      </c>
-      <c r="I14" s="53"/>
+      <c r="H14" s="72" t="s">
+        <v>108</v>
+      </c>
+      <c r="I14" s="49"/>
       <c r="J14" s="20"/>
     </row>
     <row r="15" spans="1:29" ht="47.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="112" t="s">
+      <c r="A15" s="107" t="s">
         <v>33</v>
       </c>
       <c r="B15" s="13" t="s">
         <v>36</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>75</v>
+        <v>147</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="71" t="s">
+      <c r="E15" s="67" t="s">
         <v>59</v>
       </c>
       <c r="F15" s="36" t="s">
-        <v>143</v>
-      </c>
-      <c r="G15" s="54" t="s">
-        <v>96</v>
-      </c>
-      <c r="H15" s="40" t="s">
-        <v>77</v>
-      </c>
-      <c r="I15" s="19"/>
+        <v>139</v>
+      </c>
+      <c r="G15" s="50" t="s">
+        <v>92</v>
+      </c>
+      <c r="H15" s="115" t="s">
+        <v>108</v>
+      </c>
+      <c r="I15" s="19" t="s">
+        <v>148</v>
+      </c>
       <c r="J15" s="20"/>
     </row>
     <row r="16" spans="1:29" ht="48.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="112"/>
+      <c r="A16" s="107"/>
       <c r="B16" s="13" t="s">
         <v>37</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="71" t="s">
+      <c r="E16" s="67" t="s">
         <v>59</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>143</v>
-      </c>
-      <c r="G16" s="54" t="s">
-        <v>96</v>
-      </c>
-      <c r="H16" s="40" t="s">
-        <v>77</v>
-      </c>
-      <c r="I16" s="19"/>
+        <v>139</v>
+      </c>
+      <c r="G16" s="50" t="s">
+        <v>92</v>
+      </c>
+      <c r="H16" s="115" t="s">
+        <v>108</v>
+      </c>
+      <c r="I16" s="19" t="s">
+        <v>145</v>
+      </c>
       <c r="J16" s="20"/>
     </row>
     <row r="17" spans="1:29" s="7" customFormat="1" ht="51.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="113"/>
+      <c r="A17" s="108"/>
       <c r="B17" s="14" t="s">
         <v>38</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="72" t="s">
+      <c r="E17" s="68" t="s">
         <v>59</v>
       </c>
-      <c r="F17" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="G17" s="54" t="s">
-        <v>96</v>
-      </c>
-      <c r="H17" s="41" t="s">
-        <v>77</v>
-      </c>
-      <c r="I17" s="18"/>
+      <c r="F17" s="68" t="s">
+        <v>139</v>
+      </c>
+      <c r="G17" s="50" t="s">
+        <v>92</v>
+      </c>
+      <c r="H17" s="116" t="s">
+        <v>108</v>
+      </c>
+      <c r="I17" s="18" t="s">
+        <v>146</v>
+      </c>
       <c r="J17" s="20"/>
       <c r="K17"/>
       <c r="L17"/>
@@ -2423,40 +2460,40 @@
       <c r="AC17"/>
     </row>
     <row r="18" spans="1:29" ht="33" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="114" t="s">
+      <c r="A18" s="109" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="43" t="s">
+      <c r="B18" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="43" t="s">
+      <c r="C18" s="41" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="43" t="s">
+      <c r="D18" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="44" t="s">
+      <c r="E18" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="F18" s="44" t="s">
+      <c r="F18" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="G18" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="H18" s="69" t="s">
-        <v>112</v>
-      </c>
-      <c r="I18" s="48"/>
+      <c r="G18" s="54" t="s">
+        <v>91</v>
+      </c>
+      <c r="H18" s="65" t="s">
+        <v>108</v>
+      </c>
+      <c r="I18" s="45"/>
       <c r="J18" s="20"/>
     </row>
     <row r="19" spans="1:29" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="90"/>
+      <c r="A19" s="85"/>
       <c r="B19" s="11" t="s">
         <v>44</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>19</v>
@@ -2467,17 +2504,17 @@
       <c r="F19" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G19" s="59" t="s">
-        <v>95</v>
-      </c>
-      <c r="H19" s="75" t="s">
-        <v>112</v>
+      <c r="G19" s="55" t="s">
+        <v>91</v>
+      </c>
+      <c r="H19" s="71" t="s">
+        <v>108</v>
       </c>
       <c r="I19" s="28"/>
       <c r="J19" s="20"/>
     </row>
     <row r="20" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="90"/>
+      <c r="A20" s="85"/>
       <c r="B20" s="11" t="s">
         <v>40</v>
       </c>
@@ -2493,17 +2530,17 @@
       <c r="F20" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G20" s="59" t="s">
-        <v>95</v>
-      </c>
-      <c r="H20" s="75" t="s">
-        <v>112</v>
+      <c r="G20" s="55" t="s">
+        <v>91</v>
+      </c>
+      <c r="H20" s="71" t="s">
+        <v>108</v>
       </c>
       <c r="I20" s="19"/>
       <c r="J20" s="20"/>
     </row>
     <row r="21" spans="1:29" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="90"/>
+      <c r="A21" s="85"/>
       <c r="B21" s="11" t="s">
         <v>41</v>
       </c>
@@ -2519,17 +2556,17 @@
       <c r="F21" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G21" s="59" t="s">
-        <v>95</v>
-      </c>
-      <c r="H21" s="75" t="s">
-        <v>112</v>
+      <c r="G21" s="55" t="s">
+        <v>91</v>
+      </c>
+      <c r="H21" s="71" t="s">
+        <v>108</v>
       </c>
       <c r="I21" s="19"/>
       <c r="J21" s="20"/>
     </row>
     <row r="22" spans="1:29" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="90"/>
+      <c r="A22" s="85"/>
       <c r="B22" s="11" t="s">
         <v>35</v>
       </c>
@@ -2545,19 +2582,19 @@
       <c r="F22" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G22" s="59" t="s">
-        <v>95</v>
-      </c>
-      <c r="H22" s="75" t="s">
-        <v>112</v>
+      <c r="G22" s="55" t="s">
+        <v>91</v>
+      </c>
+      <c r="H22" s="71" t="s">
+        <v>108</v>
       </c>
       <c r="I22" s="19" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="J22" s="20"/>
     </row>
     <row r="23" spans="1:29" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="90"/>
+      <c r="A23" s="85"/>
       <c r="B23" s="11" t="s">
         <v>42</v>
       </c>
@@ -2573,39 +2610,39 @@
       <c r="F23" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G23" s="59" t="s">
-        <v>95</v>
-      </c>
-      <c r="H23" s="75" t="s">
-        <v>112</v>
+      <c r="G23" s="55" t="s">
+        <v>91</v>
+      </c>
+      <c r="H23" s="71" t="s">
+        <v>108</v>
       </c>
       <c r="I23" s="27"/>
       <c r="J23" s="20"/>
     </row>
     <row r="24" spans="1:29" s="7" customFormat="1" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="91"/>
-      <c r="B24" s="50" t="s">
+      <c r="A24" s="86"/>
+      <c r="B24" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="50" t="s">
+      <c r="C24" s="46" t="s">
         <v>52</v>
       </c>
-      <c r="D24" s="50" t="s">
+      <c r="D24" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="51" t="s">
+      <c r="E24" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="F24" s="51" t="s">
+      <c r="F24" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="G24" s="60" t="s">
-        <v>95</v>
-      </c>
-      <c r="H24" s="76" t="s">
-        <v>112</v>
-      </c>
-      <c r="I24" s="53"/>
+      <c r="G24" s="56" t="s">
+        <v>91</v>
+      </c>
+      <c r="H24" s="72" t="s">
+        <v>108</v>
+      </c>
+      <c r="I24" s="49"/>
       <c r="J24" s="20"/>
       <c r="K24"/>
       <c r="L24"/>
@@ -2628,32 +2665,32 @@
       <c r="AC24"/>
     </row>
     <row r="25" spans="1:29" s="15" customFormat="1" ht="29.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="106" t="s">
+      <c r="A25" s="101" t="s">
         <v>53</v>
       </c>
-      <c r="B25" s="43" t="s">
+      <c r="B25" s="41" t="s">
         <v>55</v>
       </c>
-      <c r="C25" s="43" t="s">
+      <c r="C25" s="41" t="s">
         <v>60</v>
       </c>
-      <c r="D25" s="43" t="s">
+      <c r="D25" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="E25" s="44" t="s">
+      <c r="E25" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="F25" s="44" t="s">
+      <c r="F25" s="42" t="s">
         <v>58</v>
       </c>
-      <c r="G25" s="54" t="s">
-        <v>96</v>
-      </c>
-      <c r="H25" s="47" t="s">
-        <v>77</v>
-      </c>
-      <c r="I25" s="48" t="s">
-        <v>146</v>
+      <c r="G25" s="50" t="s">
+        <v>92</v>
+      </c>
+      <c r="H25" s="65" t="s">
+        <v>108</v>
+      </c>
+      <c r="I25" s="45" t="s">
+        <v>164</v>
       </c>
       <c r="J25"/>
       <c r="K25"/>
@@ -2677,12 +2714,12 @@
       <c r="AC25"/>
     </row>
     <row r="26" spans="1:29" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="107"/>
+      <c r="A26" s="102"/>
       <c r="B26" s="11" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>19</v>
@@ -2693,41 +2730,41 @@
       <c r="F26" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="G26" s="55" t="s">
-        <v>96</v>
-      </c>
-      <c r="H26" s="75" t="s">
-        <v>112</v>
+      <c r="G26" s="51" t="s">
+        <v>92</v>
+      </c>
+      <c r="H26" s="71" t="s">
+        <v>108</v>
       </c>
       <c r="I26" s="19" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
     </row>
     <row r="27" spans="1:29" s="17" customFormat="1" ht="55.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="108"/>
-      <c r="B27" s="50" t="s">
+      <c r="A27" s="103"/>
+      <c r="B27" s="46" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="50" t="s">
+      <c r="C27" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="D27" s="50" t="s">
+      <c r="D27" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="E27" s="51" t="s">
+      <c r="E27" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="F27" s="56" t="s">
+      <c r="F27" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="G27" s="57" t="s">
-        <v>94</v>
-      </c>
-      <c r="H27" s="76" t="s">
-        <v>112</v>
-      </c>
-      <c r="I27" s="53" t="s">
-        <v>129</v>
+      <c r="G27" s="53" t="s">
+        <v>90</v>
+      </c>
+      <c r="H27" s="72" t="s">
+        <v>108</v>
+      </c>
+      <c r="I27" s="49" t="s">
+        <v>125</v>
       </c>
       <c r="J27"/>
       <c r="K27"/>
@@ -2751,41 +2788,41 @@
       <c r="AC27"/>
     </row>
     <row r="28" spans="1:29" ht="28.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="89" t="s">
+      <c r="A28" s="84" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="43" t="s">
+      <c r="B28" s="41" t="s">
+        <v>93</v>
+      </c>
+      <c r="C28" s="41" t="s">
+        <v>98</v>
+      </c>
+      <c r="D28" s="41" t="s">
+        <v>19</v>
+      </c>
+      <c r="E28" s="42" t="s">
+        <v>32</v>
+      </c>
+      <c r="F28" s="43" t="s">
+        <v>20</v>
+      </c>
+      <c r="G28" s="44" t="s">
+        <v>89</v>
+      </c>
+      <c r="H28" s="65" t="s">
+        <v>108</v>
+      </c>
+      <c r="I28" s="45" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="29" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="85"/>
+      <c r="B29" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="C29" s="11" t="s">
         <v>97</v>
-      </c>
-      <c r="C28" s="43" t="s">
-        <v>102</v>
-      </c>
-      <c r="D28" s="43" t="s">
-        <v>19</v>
-      </c>
-      <c r="E28" s="44" t="s">
-        <v>32</v>
-      </c>
-      <c r="F28" s="45" t="s">
-        <v>20</v>
-      </c>
-      <c r="G28" s="46" t="s">
-        <v>93</v>
-      </c>
-      <c r="H28" s="69" t="s">
-        <v>112</v>
-      </c>
-      <c r="I28" s="48" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="29" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="90"/>
-      <c r="B29" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>101</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>19</v>
@@ -2797,20 +2834,20 @@
         <v>20</v>
       </c>
       <c r="G29" s="37" t="s">
-        <v>93</v>
-      </c>
-      <c r="H29" s="75" t="s">
-        <v>112</v>
+        <v>89</v>
+      </c>
+      <c r="H29" s="71" t="s">
+        <v>108</v>
       </c>
       <c r="I29" s="19"/>
     </row>
     <row r="30" spans="1:29" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="90"/>
+      <c r="A30" s="85"/>
       <c r="B30" s="11" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>19</v>
@@ -2822,20 +2859,20 @@
         <v>20</v>
       </c>
       <c r="G30" s="37" t="s">
-        <v>93</v>
-      </c>
-      <c r="H30" s="75" t="s">
-        <v>77</v>
+        <v>89</v>
+      </c>
+      <c r="H30" s="71" t="s">
+        <v>108</v>
       </c>
       <c r="I30" s="19"/>
     </row>
     <row r="31" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="90"/>
+      <c r="A31" s="85"/>
       <c r="B31" s="11" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>19</v>
@@ -2844,23 +2881,23 @@
         <v>58</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="G31" s="37" t="s">
-        <v>93</v>
-      </c>
-      <c r="H31" s="49" t="s">
-        <v>77</v>
+        <v>89</v>
+      </c>
+      <c r="H31" s="71" t="s">
+        <v>108</v>
       </c>
       <c r="I31" s="19"/>
     </row>
     <row r="32" spans="1:29" s="16" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="90"/>
+      <c r="A32" s="85"/>
       <c r="B32" s="11" t="s">
         <v>54</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="D32" s="11" t="s">
         <v>19</v>
@@ -2869,13 +2906,13 @@
         <v>32</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="G32" s="37" t="s">
-        <v>93</v>
-      </c>
-      <c r="H32" s="49" t="s">
-        <v>77</v>
+        <v>89</v>
+      </c>
+      <c r="H32" s="71" t="s">
+        <v>108</v>
       </c>
       <c r="I32" s="19"/>
       <c r="J32"/>
@@ -2900,29 +2937,31 @@
       <c r="AC32"/>
     </row>
     <row r="33" spans="1:29" s="16" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="90"/>
-      <c r="B33" s="11" t="s">
+      <c r="A33" s="85"/>
+      <c r="B33" s="117" t="s">
         <v>26</v>
       </c>
-      <c r="C33" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="D33" s="11" t="s">
+      <c r="C33" s="117" t="s">
+        <v>130</v>
+      </c>
+      <c r="D33" s="117" t="s">
         <v>19</v>
       </c>
-      <c r="E33" s="36" t="s">
+      <c r="E33" s="118" t="s">
         <v>20</v>
       </c>
-      <c r="F33" s="11" t="s">
+      <c r="F33" s="117" t="s">
         <v>58</v>
       </c>
-      <c r="G33" s="37" t="s">
-        <v>93</v>
-      </c>
-      <c r="H33" s="49" t="s">
-        <v>77</v>
-      </c>
-      <c r="I33" s="19"/>
+      <c r="G33" s="118" t="s">
+        <v>89</v>
+      </c>
+      <c r="H33" s="119" t="s">
+        <v>108</v>
+      </c>
+      <c r="I33" s="120" t="s">
+        <v>149</v>
+      </c>
       <c r="J33"/>
       <c r="K33"/>
       <c r="L33"/>
@@ -2945,12 +2984,12 @@
       <c r="AC33"/>
     </row>
     <row r="34" spans="1:29" s="16" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="90"/>
+      <c r="A34" s="85"/>
       <c r="B34" s="11" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>19</v>
@@ -2962,13 +3001,13 @@
         <v>59</v>
       </c>
       <c r="G34" s="37" t="s">
-        <v>93</v>
-      </c>
-      <c r="H34" s="75" t="s">
-        <v>112</v>
+        <v>89</v>
+      </c>
+      <c r="H34" s="71" t="s">
+        <v>108</v>
       </c>
       <c r="I34" s="19" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="J34"/>
       <c r="K34"/>
@@ -2992,12 +3031,12 @@
       <c r="AC34"/>
     </row>
     <row r="35" spans="1:29" s="16" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="90"/>
+      <c r="A35" s="85"/>
       <c r="B35" s="11" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D35" s="11" t="s">
         <v>19</v>
@@ -3009,10 +3048,10 @@
         <v>20</v>
       </c>
       <c r="G35" s="37" t="s">
-        <v>93</v>
-      </c>
-      <c r="H35" s="75" t="s">
-        <v>112</v>
+        <v>89</v>
+      </c>
+      <c r="H35" s="71" t="s">
+        <v>108</v>
       </c>
       <c r="I35" s="19"/>
       <c r="J35"/>
@@ -3037,29 +3076,29 @@
       <c r="AC35"/>
     </row>
     <row r="36" spans="1:29" s="16" customFormat="1" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="91"/>
-      <c r="B36" s="50" t="s">
-        <v>107</v>
-      </c>
-      <c r="C36" s="50" t="s">
+      <c r="A36" s="86"/>
+      <c r="B36" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="C36" s="46" t="s">
+        <v>104</v>
+      </c>
+      <c r="D36" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="E36" s="47" t="s">
+        <v>32</v>
+      </c>
+      <c r="F36" s="47" t="s">
+        <v>20</v>
+      </c>
+      <c r="G36" s="48" t="s">
+        <v>89</v>
+      </c>
+      <c r="H36" s="72" t="s">
         <v>108</v>
       </c>
-      <c r="D36" s="50" t="s">
-        <v>19</v>
-      </c>
-      <c r="E36" s="51" t="s">
-        <v>32</v>
-      </c>
-      <c r="F36" s="51" t="s">
-        <v>20</v>
-      </c>
-      <c r="G36" s="52" t="s">
-        <v>93</v>
-      </c>
-      <c r="H36" s="76" t="s">
-        <v>112</v>
-      </c>
-      <c r="I36" s="53"/>
+      <c r="I36" s="49"/>
       <c r="J36"/>
       <c r="K36"/>
       <c r="L36"/>
@@ -3107,7 +3146,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{748CED0D-D7CE-4618-A56E-B7666AE2995E}">
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.42578125" style="1" customWidth="1"/>
@@ -3121,28 +3160,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="115" t="s">
+      <c r="A1" s="110" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="79"/>
+      <c r="B1" s="111"/>
+      <c r="C1" s="111"/>
+      <c r="D1" s="111"/>
+      <c r="E1" s="111"/>
+      <c r="F1" s="111"/>
+      <c r="G1" s="75"/>
     </row>
     <row r="2" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="39" t="s">
-        <v>82</v>
-      </c>
-      <c r="B2" s="117" t="s">
-        <v>85</v>
-      </c>
-      <c r="C2" s="118"/>
-      <c r="D2" s="118"/>
-      <c r="E2" s="118"/>
-      <c r="F2" s="118"/>
-      <c r="G2" s="80"/>
+        <v>78</v>
+      </c>
+      <c r="B2" s="112" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2" s="113"/>
+      <c r="D2" s="113"/>
+      <c r="E2" s="113"/>
+      <c r="F2" s="113"/>
+      <c r="G2" s="76"/>
     </row>
     <row r="3" spans="1:8" s="26" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
@@ -3160,281 +3199,304 @@
       <c r="E3" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="77" t="s">
+      <c r="F3" s="73" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="81" t="s">
-        <v>87</v>
-      </c>
-      <c r="H3" s="78"/>
+      <c r="G3" s="77" t="s">
+        <v>83</v>
+      </c>
+      <c r="H3" s="74"/>
     </row>
     <row r="4" spans="1:8" ht="225.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="82" t="s">
+      <c r="A4" s="78" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="82" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" s="83" t="s">
+      <c r="B4" s="78" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="79" t="s">
+        <v>118</v>
+      </c>
+      <c r="D4" s="78" t="s">
+        <v>119</v>
+      </c>
+      <c r="E4" s="78" t="s">
+        <v>120</v>
+      </c>
+      <c r="F4" s="78" t="s">
+        <v>121</v>
+      </c>
+      <c r="G4" s="78" t="s">
         <v>122</v>
       </c>
-      <c r="D4" s="82" t="s">
-        <v>123</v>
-      </c>
-      <c r="E4" s="82" t="s">
-        <v>124</v>
-      </c>
-      <c r="F4" s="82" t="s">
-        <v>125</v>
-      </c>
-      <c r="G4" s="82" t="s">
+    </row>
+    <row r="5" spans="1:8" ht="143.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="78" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="78" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="79" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" s="78" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="143.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="82" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5" s="82" t="s">
-        <v>63</v>
-      </c>
-      <c r="C5" s="83" t="s">
-        <v>84</v>
-      </c>
-      <c r="D5" s="82" t="s">
-        <v>130</v>
-      </c>
-      <c r="E5" s="82" t="s">
-        <v>131</v>
-      </c>
-      <c r="F5" s="82" t="s">
-        <v>132</v>
-      </c>
-      <c r="G5" s="82" t="s">
-        <v>133</v>
+      <c r="E5" s="78" t="s">
+        <v>127</v>
+      </c>
+      <c r="F5" s="78" t="s">
+        <v>128</v>
+      </c>
+      <c r="G5" s="78" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="191.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="82" t="s">
+      <c r="A6" s="78" t="s">
         <v>64</v>
       </c>
-      <c r="B6" s="82" t="s">
+      <c r="B6" s="78" t="s">
         <v>65</v>
       </c>
-      <c r="C6" s="83" t="s">
-        <v>84</v>
-      </c>
-      <c r="D6" s="82"/>
-      <c r="E6" s="82"/>
-      <c r="F6" s="82"/>
-      <c r="G6" s="82"/>
+      <c r="C6" s="79" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" s="78" t="s">
+        <v>150</v>
+      </c>
+      <c r="E6" s="78" t="s">
+        <v>151</v>
+      </c>
+      <c r="F6" s="78" t="s">
+        <v>152</v>
+      </c>
+      <c r="G6" s="78" t="s">
+        <v>153</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="115.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="82" t="s">
+      <c r="A7" s="78" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="82" t="s">
-        <v>72</v>
-      </c>
-      <c r="C7" s="83" t="s">
-        <v>84</v>
-      </c>
-      <c r="D7" s="82"/>
-      <c r="E7" s="82"/>
-      <c r="F7" s="82"/>
-      <c r="G7" s="82"/>
+      <c r="B7" s="78" t="s">
+        <v>154</v>
+      </c>
+      <c r="C7" s="79" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="78"/>
+      <c r="E7" s="78"/>
+      <c r="F7" s="78"/>
+      <c r="G7" s="78"/>
     </row>
     <row r="8" spans="1:8" s="29" customFormat="1" ht="227.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="84" t="s">
-        <v>71</v>
-      </c>
-      <c r="B8" s="119" t="s">
+      <c r="A8" s="80" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="114" t="s">
         <v>66</v>
       </c>
-      <c r="C8" s="83" t="s">
-        <v>84</v>
-      </c>
-      <c r="D8" s="82"/>
-      <c r="E8" s="85"/>
-      <c r="F8" s="82"/>
-      <c r="G8" s="82"/>
+      <c r="C8" s="79" t="s">
+        <v>80</v>
+      </c>
+      <c r="D8" s="78"/>
+      <c r="E8" s="81"/>
+      <c r="F8" s="78"/>
+      <c r="G8" s="78"/>
     </row>
     <row r="9" spans="1:8" ht="238.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="82" t="s">
+      <c r="A9" s="78" t="s">
         <v>67</v>
       </c>
-      <c r="B9" s="119"/>
-      <c r="C9" s="83" t="s">
-        <v>84</v>
-      </c>
-      <c r="D9" s="82"/>
-      <c r="E9" s="85"/>
-      <c r="F9" s="82"/>
-      <c r="G9" s="82"/>
-    </row>
-    <row r="10" spans="1:8" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="86" t="s">
+      <c r="B9" s="114"/>
+      <c r="C9" s="79" t="s">
+        <v>80</v>
+      </c>
+      <c r="D9" s="78" t="s">
+        <v>161</v>
+      </c>
+      <c r="E9" s="26" t="s">
+        <v>162</v>
+      </c>
+      <c r="F9" s="78" t="s">
+        <v>163</v>
+      </c>
+      <c r="G9" s="78" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="145.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="78" t="s">
         <v>68</v>
       </c>
-      <c r="B10" s="119"/>
-      <c r="C10" s="86" t="s">
-        <v>84</v>
-      </c>
-      <c r="D10" s="86"/>
-      <c r="E10" s="85"/>
-      <c r="F10" s="82"/>
-      <c r="G10" s="82"/>
-    </row>
-    <row r="11" spans="1:8" ht="145.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="82" t="s">
+      <c r="B10" s="114"/>
+      <c r="C10" s="79" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="78" t="s">
+        <v>158</v>
+      </c>
+      <c r="E10" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="F10" s="78" t="s">
+        <v>160</v>
+      </c>
+      <c r="G10" s="78" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="30" customFormat="1" ht="102" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="78" t="s">
         <v>69</v>
       </c>
-      <c r="B11" s="119"/>
-      <c r="C11" s="83" t="s">
-        <v>84</v>
-      </c>
-      <c r="D11" s="82"/>
-      <c r="E11" s="85"/>
-      <c r="F11" s="82"/>
-      <c r="G11" s="82"/>
-    </row>
-    <row r="12" spans="1:8" s="30" customFormat="1" ht="102" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="82" t="s">
-        <v>70</v>
-      </c>
-      <c r="B12" s="119"/>
-      <c r="C12" s="83" t="s">
-        <v>84</v>
-      </c>
-      <c r="D12" s="82"/>
-      <c r="E12" s="85"/>
-      <c r="F12" s="82"/>
-      <c r="G12" s="82"/>
+      <c r="B11" s="114"/>
+      <c r="C11" s="79" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="78" t="s">
+        <v>155</v>
+      </c>
+      <c r="E11" s="26" t="s">
+        <v>156</v>
+      </c>
+      <c r="F11" s="78" t="s">
+        <v>157</v>
+      </c>
+      <c r="G11" s="78" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="78" t="s">
+        <v>110</v>
+      </c>
+      <c r="B12" s="78" t="s">
+        <v>113</v>
+      </c>
+      <c r="C12" s="79" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="78"/>
+      <c r="E12" s="78"/>
+      <c r="F12" s="78"/>
+      <c r="G12" s="78"/>
     </row>
     <row r="13" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="82" t="s">
+      <c r="A13" s="78" t="s">
+        <v>111</v>
+      </c>
+      <c r="B13" s="78" t="s">
         <v>114</v>
       </c>
-      <c r="B13" s="82" t="s">
+      <c r="C13" s="79" t="s">
+        <v>80</v>
+      </c>
+      <c r="D13" s="78"/>
+      <c r="E13" s="78"/>
+      <c r="F13" s="78"/>
+      <c r="G13" s="78"/>
+    </row>
+    <row r="14" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="78" t="s">
+        <v>112</v>
+      </c>
+      <c r="B14" s="78" t="s">
+        <v>115</v>
+      </c>
+      <c r="C14" s="79" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="78"/>
+      <c r="E14" s="78"/>
+      <c r="F14" s="78"/>
+      <c r="G14" s="78"/>
+    </row>
+    <row r="15" spans="1:8" ht="84" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="78" t="s">
+        <v>116</v>
+      </c>
+      <c r="B15" s="78" t="s">
         <v>117</v>
       </c>
-      <c r="C13" s="83" t="s">
-        <v>84</v>
-      </c>
-      <c r="D13" s="82"/>
-      <c r="E13" s="82"/>
-      <c r="F13" s="82"/>
-      <c r="G13" s="82"/>
-    </row>
-    <row r="14" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="82" t="s">
-        <v>115</v>
-      </c>
-      <c r="B14" s="82" t="s">
-        <v>118</v>
-      </c>
-      <c r="C14" s="83" t="s">
-        <v>84</v>
-      </c>
-      <c r="D14" s="82"/>
-      <c r="E14" s="82"/>
-      <c r="F14" s="82"/>
-      <c r="G14" s="82"/>
-    </row>
-    <row r="15" spans="1:8" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="82" t="s">
-        <v>116</v>
-      </c>
-      <c r="B15" s="82" t="s">
-        <v>119</v>
-      </c>
-      <c r="C15" s="83" t="s">
-        <v>84</v>
-      </c>
-      <c r="D15" s="82"/>
-      <c r="E15" s="82"/>
-      <c r="F15" s="82"/>
-      <c r="G15" s="82"/>
-    </row>
-    <row r="16" spans="1:8" ht="84" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="82" t="s">
-        <v>120</v>
-      </c>
-      <c r="B16" s="82" t="s">
-        <v>121</v>
-      </c>
-      <c r="C16" s="82"/>
-      <c r="D16" s="82"/>
-      <c r="E16" s="82"/>
-      <c r="F16" s="82"/>
-      <c r="G16" s="82"/>
-    </row>
-    <row r="17" spans="1:7" ht="99.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="82"/>
-      <c r="B17" s="82"/>
-      <c r="C17" s="82"/>
-      <c r="D17" s="82"/>
-      <c r="E17" s="82"/>
-      <c r="F17" s="82"/>
-      <c r="G17" s="82"/>
-    </row>
-    <row r="18" spans="1:7" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C15" s="78"/>
+      <c r="D15" s="78"/>
+      <c r="E15" s="78"/>
+      <c r="F15" s="78"/>
+      <c r="G15" s="78"/>
+    </row>
+    <row r="16" spans="1:8" ht="99.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="78"/>
+      <c r="B16" s="78"/>
+      <c r="C16" s="78"/>
+      <c r="D16" s="78"/>
+      <c r="E16" s="78"/>
+      <c r="F16" s="78"/>
+      <c r="G16" s="78"/>
+    </row>
+    <row r="17" spans="1:6" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="21"/>
+      <c r="F17" s="22"/>
+    </row>
+    <row r="18" spans="1:6" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="21"/>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:7" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="78" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="21"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:7" ht="78" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="21"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:7" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="21"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:7" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="21"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:7" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="21"/>
       <c r="F23" s="22"/>
     </row>
-    <row r="24" spans="1:7" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="21"/>
       <c r="F24" s="22"/>
     </row>
-    <row r="25" spans="1:7" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="21"/>
       <c r="F25" s="22"/>
     </row>
-    <row r="26" spans="1:7" ht="101.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="21"/>
       <c r="F26" s="22"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="21"/>
       <c r="F27" s="22"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="21"/>
       <c r="F28" s="22"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="21"/>
       <c r="F29" s="22"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="21"/>
       <c r="F30" s="22"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="21"/>
       <c r="F31" s="22"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="21"/>
       <c r="F32" s="22"/>
     </row>
@@ -3477,16 +3539,12 @@
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="21"/>
       <c r="F42" s="22"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="21"/>
-      <c r="F43" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B8:B12"/>
+    <mergeCell ref="B8:B11"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{B6652C4F-D602-413E-8A18-C0965E86E210}"/>
@@ -3753,6 +3811,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="ff8a4b2e-b0c8-4039-a689-d1a7f36f4382">
@@ -3762,15 +3829,6 @@
     <Notes xmlns="ff8a4b2e-b0c8-4039-a689-d1a7f36f4382" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3793,6 +3851,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8F3069D-89E7-4007-93BF-1DB2942FF756}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76F271AB-EFB2-4823-A2F0-9F2289E658DB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3803,12 +3869,4 @@
     <ds:schemaRef ds:uri="f716dd8a-49a0-4c40-b209-038e1651b548"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8F3069D-89E7-4007-93BF-1DB2942FF756}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>